<commit_message>
Updated City/State respondent order
</commit_message>
<xml_diff>
--- a/June 2025 SATS+ Output.xlsx
+++ b/June 2025 SATS+ Output.xlsx
@@ -1303,21 +1303,21 @@
       </c>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="n">
-        <v>8760</v>
+        <v>7181</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>jxn419t3wxgf43ge</t>
+          <t>05tev9d85zfq9uzd</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>06/22/2025 20:50</t>
+          <t>06/22/2025 07:49</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>qualified,/D Apollo Destination 1/Philadelphia__Pennsylvania,20250622_14:03_v148,/D Apollo State 1/Illinois,/Unemployed and Retired/MSkJW,/Quota by US Census Region/Origin Region West,Illinois,Philadelphia__Pennsylvania</t>
+          <t>qualified,Nevada,/Quota by US Census Region/Origin Region South,/D Apollo State 1/Nevada,/Unemployed and Retired/cJ2Bp,Montreal_Quebec,20250617_14:32_v146,/D Apollo Destination 1/Montreal_Quebec</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -1327,34 +1327,34 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="J3" t="n">
-        <v>1982</v>
+        <v>1954</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Arizona</t>
+          <t>Maryland</t>
         </is>
       </c>
       <c r="L3" t="n">
-        <v>86440</v>
+        <v>21921</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>$80,000 to $99,999</t>
+          <t>$150,000 to $199,999</t>
         </is>
       </c>
       <c r="N3" t="inlineStr"/>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Rural area</t>
+          <t>Small town (not near an urban area)</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>Employed (full-time)</t>
+          <t>Employed (part-time)</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
@@ -1364,62 +1364,30 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="S3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="T3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="U3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="V3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="W3" t="inlineStr">
-        <is>
-          <t>Psychological issues</t>
-        </is>
-      </c>
-      <c r="X3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Y3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Z3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr"/>
+      <c r="T3" t="inlineStr"/>
+      <c r="U3" t="inlineStr"/>
+      <c r="V3" t="inlineStr"/>
+      <c r="W3" t="inlineStr"/>
+      <c r="X3" t="inlineStr"/>
+      <c r="Y3" t="inlineStr"/>
+      <c r="Z3" t="inlineStr"/>
       <c r="AA3" t="inlineStr">
         <is>
-          <t>Hispanic/Latino</t>
+          <t>White</t>
         </is>
       </c>
       <c r="AB3" t="inlineStr">
         <is>
-          <t>Completed graduate degree</t>
+          <t>Some college</t>
         </is>
       </c>
       <c r="AC3" t="inlineStr">
         <is>
-          <t>Single</t>
+          <t>Married</t>
         </is>
       </c>
       <c r="AD3" t="inlineStr"/>
@@ -1433,7 +1401,7 @@
       </c>
       <c r="AI3" t="inlineStr">
         <is>
-          <t>Libertarian</t>
+          <t>Unaffiliated with a political party</t>
         </is>
       </c>
       <c r="AJ3" t="inlineStr"/>
@@ -1444,7 +1412,7 @@
       </c>
       <c r="AL3" t="inlineStr">
         <is>
-          <t>Unfamiliar</t>
+          <t>Neutral (neither familiar nor unfamiliar)</t>
         </is>
       </c>
       <c r="AM3" t="inlineStr">
@@ -1464,7 +1432,7 @@
       </c>
       <c r="AP3" t="inlineStr">
         <is>
-          <t>Neutral – neither good nor poor</t>
+          <t>Slightly good</t>
         </is>
       </c>
       <c r="AQ3" t="inlineStr">
@@ -1479,7 +1447,7 @@
       </c>
       <c r="AS3" t="inlineStr">
         <is>
-          <t>Slightly good</t>
+          <t>Good</t>
         </is>
       </c>
       <c r="AT3" t="inlineStr">
@@ -1489,7 +1457,7 @@
       </c>
       <c r="AU3" t="inlineStr">
         <is>
-          <t>Neutral – neither good nor poor</t>
+          <t>Good</t>
         </is>
       </c>
       <c r="AV3" t="inlineStr">
@@ -1499,12 +1467,12 @@
       </c>
       <c r="AW3" t="inlineStr">
         <is>
-          <t>Slightly good</t>
+          <t>Good</t>
         </is>
       </c>
       <c r="AX3" t="inlineStr">
         <is>
-          <t>Neutral – neither good nor poor</t>
+          <t>Good</t>
         </is>
       </c>
       <c r="AY3" t="inlineStr">
@@ -1524,57 +1492,57 @@
       </c>
       <c r="BB3" t="inlineStr">
         <is>
-          <t>Slightly poor</t>
+          <t>Slightly good</t>
         </is>
       </c>
       <c r="BC3" t="inlineStr">
         <is>
+          <t>Slightly good</t>
+        </is>
+      </c>
+      <c r="BD3" t="inlineStr">
+        <is>
+          <t>Neutral – neither good nor poor</t>
+        </is>
+      </c>
+      <c r="BE3" t="inlineStr">
+        <is>
+          <t>Slightly good</t>
+        </is>
+      </c>
+      <c r="BF3" t="inlineStr">
+        <is>
+          <t>Neutral – neither good nor poor</t>
+        </is>
+      </c>
+      <c r="BG3" t="inlineStr">
+        <is>
+          <t>Neutral – neither good nor poor</t>
+        </is>
+      </c>
+      <c r="BH3" t="inlineStr">
+        <is>
+          <t>Slightly good</t>
+        </is>
+      </c>
+      <c r="BI3" t="inlineStr">
+        <is>
+          <t>Slightly good</t>
+        </is>
+      </c>
+      <c r="BJ3" t="inlineStr">
+        <is>
           <t>Good</t>
         </is>
       </c>
-      <c r="BD3" t="inlineStr">
-        <is>
-          <t>Good</t>
-        </is>
-      </c>
-      <c r="BE3" t="inlineStr">
-        <is>
-          <t>Good</t>
-        </is>
-      </c>
-      <c r="BF3" t="inlineStr">
-        <is>
-          <t>Neutral – neither good nor poor</t>
-        </is>
-      </c>
-      <c r="BG3" t="inlineStr">
-        <is>
-          <t>Good</t>
-        </is>
-      </c>
-      <c r="BH3" t="inlineStr">
-        <is>
-          <t>Slightly good</t>
-        </is>
-      </c>
-      <c r="BI3" t="inlineStr">
-        <is>
-          <t>Good</t>
-        </is>
-      </c>
-      <c r="BJ3" t="inlineStr">
-        <is>
-          <t>Slightly good</t>
-        </is>
-      </c>
       <c r="BK3" t="inlineStr">
         <is>
-          <t>Good</t>
+          <t>Slightly good</t>
         </is>
       </c>
       <c r="BL3" t="inlineStr">
         <is>
-          <t>Good</t>
+          <t>Neutral – neither good nor poor</t>
         </is>
       </c>
       <c r="BM3" t="inlineStr">
@@ -1584,7 +1552,7 @@
       </c>
       <c r="BN3" t="inlineStr">
         <is>
-          <t>Slightly good</t>
+          <t>Neutral – neither good nor poor</t>
         </is>
       </c>
       <c r="BO3" t="inlineStr">
@@ -1607,16 +1575,16 @@
       </c>
       <c r="BS3" t="inlineStr">
         <is>
-          <t>Very welcoming</t>
+          <t>Slightly welcoming</t>
         </is>
       </c>
       <c r="BT3" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="BU3" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="BV3" t="inlineStr">
         <is>
@@ -1635,20 +1603,22 @@
       </c>
       <c r="BY3" t="inlineStr">
         <is>
-          <t>Strongly agree</t>
+          <t>Agree</t>
         </is>
       </c>
       <c r="BZ3" t="inlineStr">
         <is>
-          <t>Slightly appealing</t>
-        </is>
-      </c>
-      <c r="CA3" t="n">
-        <v>7</v>
+          <t>Neutral (neither appealing nor unappealing)</t>
+        </is>
+      </c>
+      <c r="CA3" t="inlineStr">
+        <is>
+          <t>5 – Average accessibility</t>
+        </is>
       </c>
       <c r="CB3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>I’ve been there, done that</t>
         </is>
       </c>
       <c r="CC3" t="inlineStr">
@@ -1683,7 +1653,7 @@
       </c>
       <c r="CI3" t="inlineStr">
         <is>
-          <t>It’s too far away/too hard to get to</t>
+          <t>-</t>
         </is>
       </c>
       <c r="CJ3" t="inlineStr">
@@ -1693,12 +1663,12 @@
       </c>
       <c r="CK3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>I don't like the weather there</t>
         </is>
       </c>
       <c r="CL3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>The destination is just not on my radar</t>
         </is>
       </c>
       <c r="CM3" t="inlineStr">
@@ -1740,21 +1710,21 @@
       </c>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="n">
-        <v>7181</v>
+        <v>1861</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>05tev9d85zfq9uzd</t>
+          <t>89mv39j4g4w2tmfn</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>06/22/2025 07:49</t>
+          <t>06/18/2025 16:45</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>qualified,Nevada,/Quota by US Census Region/Origin Region South,/D Apollo State 1/Nevada,/Unemployed and Retired/cJ2Bp,Montreal_Quebec,20250617_14:32_v146,/D Apollo Destination 1/Montreal_Quebec</t>
+          <t>qualified,Atlantic_City__New_Jersey,/Quota by US Census Region/Origin Region South,/D Apollo Destination 1/Atlantic_City__New_Jersey,/D Apollo State 1/Louisiana,20250617_14:32_v146,Louisiana,/Unemployed and Retired/MSkJW</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -1764,34 +1734,34 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="J4" t="n">
-        <v>1954</v>
+        <v>1967</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Maryland</t>
+          <t>North Carolina</t>
         </is>
       </c>
       <c r="L4" t="n">
-        <v>21921</v>
+        <v>27127</v>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>$150,000 to $199,999</t>
+          <t>$30,000 to $49,999</t>
         </is>
       </c>
       <c r="N4" t="inlineStr"/>
       <c r="O4" t="inlineStr">
         <is>
-          <t>Small town (not near an urban area)</t>
+          <t>Large city (urban area)</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>Employed (part-time)</t>
+          <t>Employed (full-time)</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
@@ -1819,7 +1789,7 @@
       </c>
       <c r="AB4" t="inlineStr">
         <is>
-          <t>Some college</t>
+          <t>High school graduate</t>
         </is>
       </c>
       <c r="AC4" t="inlineStr">
@@ -1838,7 +1808,7 @@
       </c>
       <c r="AI4" t="inlineStr">
         <is>
-          <t>Unaffiliated with a political party</t>
+          <t>I prefer not to answer</t>
         </is>
       </c>
       <c r="AJ4" t="inlineStr"/>
@@ -1849,17 +1819,17 @@
       </c>
       <c r="AL4" t="inlineStr">
         <is>
-          <t>Neutral (neither familiar nor unfamiliar)</t>
+          <t>Totally unfamiliar</t>
         </is>
       </c>
       <c r="AM4" t="inlineStr">
         <is>
-          <t>Unlikely</t>
+          <t>Extremely unlikely</t>
         </is>
       </c>
       <c r="AN4" t="inlineStr">
         <is>
-          <t>Slightly good</t>
+          <t>Neutral – neither good nor poor</t>
         </is>
       </c>
       <c r="AO4" t="inlineStr">
@@ -1869,7 +1839,7 @@
       </c>
       <c r="AP4" t="inlineStr">
         <is>
-          <t>Slightly good</t>
+          <t>Neutral – neither good nor poor</t>
         </is>
       </c>
       <c r="AQ4" t="inlineStr">
@@ -1884,42 +1854,42 @@
       </c>
       <c r="AS4" t="inlineStr">
         <is>
-          <t>Good</t>
+          <t>Neutral – neither good nor poor</t>
         </is>
       </c>
       <c r="AT4" t="inlineStr">
         <is>
-          <t>Good</t>
+          <t>Neutral – neither good nor poor</t>
         </is>
       </c>
       <c r="AU4" t="inlineStr">
         <is>
-          <t>Good</t>
+          <t>Neutral – neither good nor poor</t>
         </is>
       </c>
       <c r="AV4" t="inlineStr">
         <is>
-          <t>Good</t>
+          <t>Neutral – neither good nor poor</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>Good</t>
+          <t>Neutral – neither good nor poor</t>
         </is>
       </c>
       <c r="AX4" t="inlineStr">
         <is>
-          <t>Good</t>
+          <t>Neutral – neither good nor poor</t>
         </is>
       </c>
       <c r="AY4" t="inlineStr">
         <is>
-          <t>Slightly good</t>
+          <t>Neutral – neither good nor poor</t>
         </is>
       </c>
       <c r="AZ4" t="inlineStr">
         <is>
-          <t>Good</t>
+          <t>Neutral – neither good nor poor</t>
         </is>
       </c>
       <c r="BA4" t="inlineStr">
@@ -1929,12 +1899,12 @@
       </c>
       <c r="BB4" t="inlineStr">
         <is>
-          <t>Slightly good</t>
+          <t>Neutral – neither good nor poor</t>
         </is>
       </c>
       <c r="BC4" t="inlineStr">
         <is>
-          <t>Slightly good</t>
+          <t>Neutral – neither good nor poor</t>
         </is>
       </c>
       <c r="BD4" t="inlineStr">
@@ -1944,7 +1914,7 @@
       </c>
       <c r="BE4" t="inlineStr">
         <is>
-          <t>Slightly good</t>
+          <t>Neutral – neither good nor poor</t>
         </is>
       </c>
       <c r="BF4" t="inlineStr">
@@ -1959,22 +1929,22 @@
       </c>
       <c r="BH4" t="inlineStr">
         <is>
-          <t>Slightly good</t>
+          <t>Neutral – neither good nor poor</t>
         </is>
       </c>
       <c r="BI4" t="inlineStr">
         <is>
-          <t>Slightly good</t>
+          <t>Neutral – neither good nor poor</t>
         </is>
       </c>
       <c r="BJ4" t="inlineStr">
         <is>
-          <t>Good</t>
+          <t>Neutral – neither good nor poor</t>
         </is>
       </c>
       <c r="BK4" t="inlineStr">
         <is>
-          <t>Slightly good</t>
+          <t>Neutral – neither good nor poor</t>
         </is>
       </c>
       <c r="BL4" t="inlineStr">
@@ -1984,7 +1954,7 @@
       </c>
       <c r="BM4" t="inlineStr">
         <is>
-          <t>Slightly good</t>
+          <t>Neutral – neither good nor poor</t>
         </is>
       </c>
       <c r="BN4" t="inlineStr">
@@ -1994,68 +1964,72 @@
       </c>
       <c r="BO4" t="inlineStr">
         <is>
-          <t>Slightly appealing</t>
+          <t>Extremely unappealing</t>
         </is>
       </c>
       <c r="BP4" t="inlineStr">
         <is>
-          <t>Appealing</t>
+          <t>Extremely unappealing</t>
         </is>
       </c>
       <c r="BQ4" t="inlineStr">
         <is>
-          <t>Unchanged (neither more nor less popular)</t>
-        </is>
-      </c>
-      <c r="BR4" t="n">
-        <v>7</v>
+          <t>I don’t know</t>
+        </is>
+      </c>
+      <c r="BR4" t="inlineStr">
+        <is>
+          <t>0 - NOT AT ALL UNIQUE</t>
+        </is>
       </c>
       <c r="BS4" t="inlineStr">
         <is>
-          <t>Slightly welcoming</t>
+          <t>Neutral (neither welcoming nor unwelcoming)</t>
         </is>
       </c>
       <c r="BT4" t="inlineStr">
         <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="BU4" t="n">
-        <v>3</v>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="BU4" t="inlineStr">
+        <is>
+          <t>0 - NOT AT ALL MOTIVATED</t>
+        </is>
       </c>
       <c r="BV4" t="inlineStr">
         <is>
+          <t>I don’t know</t>
+        </is>
+      </c>
+      <c r="BW4" t="inlineStr">
+        <is>
           <t>No</t>
         </is>
       </c>
-      <c r="BW4" t="inlineStr">
+      <c r="BX4" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="BX4" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
       <c r="BY4" t="inlineStr">
         <is>
-          <t>Agree</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="BZ4" t="inlineStr">
         <is>
-          <t>Neutral (neither appealing nor unappealing)</t>
+          <t>Extremely unappealing</t>
         </is>
       </c>
       <c r="CA4" t="inlineStr">
         <is>
-          <t>5 – Average accessibility</t>
+          <t>0 – Far below average accessibility</t>
         </is>
       </c>
       <c r="CB4" t="inlineStr">
         <is>
-          <t>I’ve been there, done that</t>
+          <t>-</t>
         </is>
       </c>
       <c r="CC4" t="inlineStr">
@@ -2100,12 +2074,12 @@
       </c>
       <c r="CK4" t="inlineStr">
         <is>
-          <t>I don't like the weather there</t>
+          <t>-</t>
         </is>
       </c>
       <c r="CL4" t="inlineStr">
         <is>
-          <t>The destination is just not on my radar</t>
+          <t>-</t>
         </is>
       </c>
       <c r="CM4" t="inlineStr">
@@ -2115,7 +2089,7 @@
       </c>
       <c r="CN4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>NONE OF THESE</t>
         </is>
       </c>
       <c r="CO4" t="inlineStr">
@@ -2147,21 +2121,21 @@
       </c>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="n">
-        <v>7181</v>
+        <v>6602</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>05tev9d85zfq9uzd</t>
+          <t>vpyqrgreay8g67gq</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>06/22/2025 07:49</t>
+          <t>06/21/2025 23:05</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>qualified,Nevada,/Quota by US Census Region/Origin Region South,/D Apollo State 1/Nevada,/Unemployed and Retired/cJ2Bp,Montreal_Quebec,20250617_14:32_v146,/D Apollo Destination 1/Montreal_Quebec</t>
+          <t>qualified,/D Apollo Destination 1/San_Diego__California,San_Diego__California,/Quota by US Census Region/Origin Region West,/Unemployed and Retired/cJ2Bp,20250617_14:32_v146,Alabama,/D Apollo State 1/Alabama</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -2171,29 +2145,29 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="J5" t="n">
-        <v>1954</v>
+        <v>1967</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Maryland</t>
+          <t>California</t>
         </is>
       </c>
       <c r="L5" t="n">
-        <v>21921</v>
+        <v>94509</v>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>$150,000 to $199,999</t>
+          <t>$50,000 to $79,999</t>
         </is>
       </c>
       <c r="N5" t="inlineStr"/>
       <c r="O5" t="inlineStr">
         <is>
-          <t>Small town (not near an urban area)</t>
+          <t>Suburban area</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
@@ -2221,17 +2195,17 @@
       <c r="Z5" t="inlineStr"/>
       <c r="AA5" t="inlineStr">
         <is>
-          <t>White</t>
+          <t>Hispanic/Latino</t>
         </is>
       </c>
       <c r="AB5" t="inlineStr">
         <is>
-          <t>Some college</t>
+          <t>Some graduate school</t>
         </is>
       </c>
       <c r="AC5" t="inlineStr">
         <is>
-          <t>Married</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="AD5" t="inlineStr"/>
@@ -2245,7 +2219,7 @@
       </c>
       <c r="AI5" t="inlineStr">
         <is>
-          <t>Unaffiliated with a political party</t>
+          <t>Democratic</t>
         </is>
       </c>
       <c r="AJ5" t="inlineStr"/>
@@ -2261,32 +2235,32 @@
       </c>
       <c r="AM5" t="inlineStr">
         <is>
-          <t>Unlikely</t>
+          <t>Neutral (neither likely nor unlikely)</t>
         </is>
       </c>
       <c r="AN5" t="inlineStr">
         <is>
-          <t>Slightly good</t>
+          <t>Good</t>
         </is>
       </c>
       <c r="AO5" t="inlineStr">
         <is>
-          <t>Slightly good</t>
+          <t>Neutral – neither good nor poor</t>
         </is>
       </c>
       <c r="AP5" t="inlineStr">
         <is>
-          <t>Slightly good</t>
+          <t>Good</t>
         </is>
       </c>
       <c r="AQ5" t="inlineStr">
         <is>
-          <t>Slightly good</t>
+          <t>Good</t>
         </is>
       </c>
       <c r="AR5" t="inlineStr">
         <is>
-          <t>Extremely good</t>
+          <t>Good</t>
         </is>
       </c>
       <c r="AS5" t="inlineStr">
@@ -2296,109 +2270,109 @@
       </c>
       <c r="AT5" t="inlineStr">
         <is>
+          <t>Slightly good</t>
+        </is>
+      </c>
+      <c r="AU5" t="inlineStr">
+        <is>
+          <t>Slightly good</t>
+        </is>
+      </c>
+      <c r="AV5" t="inlineStr">
+        <is>
+          <t>Slightly good</t>
+        </is>
+      </c>
+      <c r="AW5" t="inlineStr">
+        <is>
           <t>Good</t>
         </is>
       </c>
-      <c r="AU5" t="inlineStr">
-        <is>
-          <t>Extremely good</t>
-        </is>
-      </c>
-      <c r="AV5" t="inlineStr">
-        <is>
-          <t>Slightly good</t>
-        </is>
-      </c>
-      <c r="AW5" t="inlineStr">
-        <is>
-          <t>Slightly good</t>
-        </is>
-      </c>
       <c r="AX5" t="inlineStr">
         <is>
+          <t>Slightly good</t>
+        </is>
+      </c>
+      <c r="AY5" t="inlineStr">
+        <is>
+          <t>Slightly good</t>
+        </is>
+      </c>
+      <c r="AZ5" t="inlineStr">
+        <is>
+          <t>Neutral – neither good nor poor</t>
+        </is>
+      </c>
+      <c r="BA5" t="inlineStr">
+        <is>
+          <t>Slightly good</t>
+        </is>
+      </c>
+      <c r="BB5" t="inlineStr">
+        <is>
+          <t>Neutral – neither good nor poor</t>
+        </is>
+      </c>
+      <c r="BC5" t="inlineStr">
+        <is>
           <t>Good</t>
         </is>
       </c>
-      <c r="AY5" t="inlineStr">
+      <c r="BD5" t="inlineStr">
+        <is>
+          <t>Slightly good</t>
+        </is>
+      </c>
+      <c r="BE5" t="inlineStr">
+        <is>
+          <t>Slightly good</t>
+        </is>
+      </c>
+      <c r="BF5" t="inlineStr">
+        <is>
+          <t>Neutral – neither good nor poor</t>
+        </is>
+      </c>
+      <c r="BG5" t="inlineStr">
+        <is>
+          <t>Slightly good</t>
+        </is>
+      </c>
+      <c r="BH5" t="inlineStr">
         <is>
           <t>Good</t>
         </is>
       </c>
-      <c r="AZ5" t="inlineStr">
+      <c r="BI5" t="inlineStr">
+        <is>
+          <t>Slightly good</t>
+        </is>
+      </c>
+      <c r="BJ5" t="inlineStr">
+        <is>
+          <t>Slightly good</t>
+        </is>
+      </c>
+      <c r="BK5" t="inlineStr">
         <is>
           <t>Good</t>
         </is>
       </c>
-      <c r="BA5" t="inlineStr">
+      <c r="BL5" t="inlineStr">
+        <is>
+          <t>Slightly good</t>
+        </is>
+      </c>
+      <c r="BM5" t="inlineStr">
         <is>
           <t>Good</t>
         </is>
       </c>
-      <c r="BB5" t="inlineStr">
+      <c r="BN5" t="inlineStr">
         <is>
           <t>Good</t>
         </is>
       </c>
-      <c r="BC5" t="inlineStr">
-        <is>
-          <t>Extremely good</t>
-        </is>
-      </c>
-      <c r="BD5" t="inlineStr">
-        <is>
-          <t>Good</t>
-        </is>
-      </c>
-      <c r="BE5" t="inlineStr">
-        <is>
-          <t>Good</t>
-        </is>
-      </c>
-      <c r="BF5" t="inlineStr">
-        <is>
-          <t>Good</t>
-        </is>
-      </c>
-      <c r="BG5" t="inlineStr">
-        <is>
-          <t>Slightly good</t>
-        </is>
-      </c>
-      <c r="BH5" t="inlineStr">
-        <is>
-          <t>Slightly good</t>
-        </is>
-      </c>
-      <c r="BI5" t="inlineStr">
-        <is>
-          <t>Extremely good</t>
-        </is>
-      </c>
-      <c r="BJ5" t="inlineStr">
-        <is>
-          <t>Slightly good</t>
-        </is>
-      </c>
-      <c r="BK5" t="inlineStr">
-        <is>
-          <t>Good</t>
-        </is>
-      </c>
-      <c r="BL5" t="inlineStr">
-        <is>
-          <t>Neutral – neither good nor poor</t>
-        </is>
-      </c>
-      <c r="BM5" t="inlineStr">
-        <is>
-          <t>Slightly good</t>
-        </is>
-      </c>
-      <c r="BN5" t="inlineStr">
-        <is>
-          <t>Good</t>
-        </is>
-      </c>
       <c r="BO5" t="inlineStr">
         <is>
           <t>Appealing</t>
@@ -2411,11 +2385,11 @@
       </c>
       <c r="BQ5" t="inlineStr">
         <is>
-          <t>Unchanged (neither more nor less popular)</t>
+          <t>More popular</t>
         </is>
       </c>
       <c r="BR5" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="BS5" t="inlineStr">
         <is>
@@ -2424,7 +2398,7 @@
       </c>
       <c r="BT5" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="BU5" t="n">
@@ -2452,90 +2426,38 @@
       </c>
       <c r="BZ5" t="inlineStr">
         <is>
-          <t>Appealing</t>
+          <t>Slightly appealing</t>
         </is>
       </c>
       <c r="CA5" t="n">
         <v>7</v>
       </c>
-      <c r="CB5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="CC5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="CD5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="CE5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="CF5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="CG5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="CH5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="CI5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="CJ5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="CK5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="CL5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="CM5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="CN5" t="inlineStr">
-        <is>
-          <t>NONE OF THESE</t>
-        </is>
-      </c>
+      <c r="CB5" t="inlineStr"/>
+      <c r="CC5" t="inlineStr"/>
+      <c r="CD5" t="inlineStr"/>
+      <c r="CE5" t="inlineStr"/>
+      <c r="CF5" t="inlineStr"/>
+      <c r="CG5" t="inlineStr"/>
+      <c r="CH5" t="inlineStr"/>
+      <c r="CI5" t="inlineStr"/>
+      <c r="CJ5" t="inlineStr"/>
+      <c r="CK5" t="inlineStr"/>
+      <c r="CL5" t="inlineStr"/>
+      <c r="CM5" t="inlineStr"/>
+      <c r="CN5" t="inlineStr"/>
       <c r="CO5" t="inlineStr">
         <is>
-          <t>Neither Agree nor Disagree</t>
+          <t>Agree</t>
         </is>
       </c>
       <c r="CP5" t="inlineStr">
         <is>
-          <t>Neither Agree nor Disagree</t>
+          <t>Agree</t>
         </is>
       </c>
       <c r="CQ5" t="inlineStr">
         <is>
-          <t>Moderately connected</t>
+          <t>Slightly connected</t>
         </is>
       </c>
     </row>
@@ -2552,21 +2474,21 @@
       </c>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="n">
-        <v>1861</v>
+        <v>9072</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>89mv39j4g4w2tmfn</t>
+          <t>6fkwnqvqaguewt8c</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>06/18/2025 16:45</t>
+          <t>06/23/2025 01:28</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>qualified,Atlantic_City__New_Jersey,/Quota by US Census Region/Origin Region South,/D Apollo Destination 1/Atlantic_City__New_Jersey,/D Apollo State 1/Louisiana,20250617_14:32_v146,Louisiana,/Unemployed and Retired/MSkJW</t>
+          <t>qualified,Georgia,20250622_14:03_v148,/D Apollo Destination 1/Nashville__Tennessee,/D Apollo State 1/Georgia,/Unemployed and Retired/cJ2Bp,Nashville__Tennessee,/Quota by US Census Region/Origin Region Midwest</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -2580,30 +2502,30 @@
         </is>
       </c>
       <c r="J6" t="n">
-        <v>1967</v>
+        <v>1969</v>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>North Carolina</t>
+          <t>Ohio</t>
         </is>
       </c>
       <c r="L6" t="n">
-        <v>27127</v>
+        <v>44641</v>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>$30,000 to $49,999</t>
+          <t>$100,000 to $124,999</t>
         </is>
       </c>
       <c r="N6" t="inlineStr"/>
       <c r="O6" t="inlineStr">
         <is>
-          <t>Large city (urban area)</t>
+          <t>Suburban area</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>Employed (full-time)</t>
+          <t>Employed (part-time)</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
@@ -2626,7 +2548,7 @@
       <c r="Z6" t="inlineStr"/>
       <c r="AA6" t="inlineStr">
         <is>
-          <t>White</t>
+          <t>Native Hawaiian/Pacific Islander</t>
         </is>
       </c>
       <c r="AB6" t="inlineStr">
@@ -2661,12 +2583,12 @@
       </c>
       <c r="AL6" t="inlineStr">
         <is>
-          <t>Totally unfamiliar</t>
+          <t>Unfamiliar</t>
         </is>
       </c>
       <c r="AM6" t="inlineStr">
         <is>
-          <t>Extremely unlikely</t>
+          <t>Neutral (neither likely nor unlikely)</t>
         </is>
       </c>
       <c r="AN6" t="inlineStr">
@@ -2806,12 +2728,12 @@
       </c>
       <c r="BO6" t="inlineStr">
         <is>
-          <t>Extremely unappealing</t>
+          <t>Slightly appealing</t>
         </is>
       </c>
       <c r="BP6" t="inlineStr">
         <is>
-          <t>Extremely unappealing</t>
+          <t>Neutral (neither appealing nor unappealing)</t>
         </is>
       </c>
       <c r="BQ6" t="inlineStr">
@@ -2819,10 +2741,8 @@
           <t>I don’t know</t>
         </is>
       </c>
-      <c r="BR6" t="inlineStr">
-        <is>
-          <t>0 - NOT AT ALL UNIQUE</t>
-        </is>
+      <c r="BR6" t="n">
+        <v>5</v>
       </c>
       <c r="BS6" t="inlineStr">
         <is>
@@ -2831,17 +2751,15 @@
       </c>
       <c r="BT6" t="inlineStr">
         <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="BU6" t="inlineStr">
-        <is>
-          <t>0 - NOT AT ALL MOTIVATED</t>
-        </is>
+          <t>A-</t>
+        </is>
+      </c>
+      <c r="BU6" t="n">
+        <v>4</v>
       </c>
       <c r="BV6" t="inlineStr">
         <is>
-          <t>I don’t know</t>
+          <t>No</t>
         </is>
       </c>
       <c r="BW6" t="inlineStr">
@@ -2861,79 +2779,25 @@
       </c>
       <c r="BZ6" t="inlineStr">
         <is>
-          <t>Extremely unappealing</t>
-        </is>
-      </c>
-      <c r="CA6" t="inlineStr">
-        <is>
-          <t>0 – Far below average accessibility</t>
-        </is>
-      </c>
-      <c r="CB6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="CC6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="CD6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="CE6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="CF6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="CG6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="CH6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="CI6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="CJ6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="CK6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="CL6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="CM6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="CN6" t="inlineStr">
-        <is>
-          <t>NONE OF THESE</t>
-        </is>
-      </c>
+          <t>Neutral (neither appealing nor unappealing)</t>
+        </is>
+      </c>
+      <c r="CA6" t="n">
+        <v>7</v>
+      </c>
+      <c r="CB6" t="inlineStr"/>
+      <c r="CC6" t="inlineStr"/>
+      <c r="CD6" t="inlineStr"/>
+      <c r="CE6" t="inlineStr"/>
+      <c r="CF6" t="inlineStr"/>
+      <c r="CG6" t="inlineStr"/>
+      <c r="CH6" t="inlineStr"/>
+      <c r="CI6" t="inlineStr"/>
+      <c r="CJ6" t="inlineStr"/>
+      <c r="CK6" t="inlineStr"/>
+      <c r="CL6" t="inlineStr"/>
+      <c r="CM6" t="inlineStr"/>
+      <c r="CN6" t="inlineStr"/>
       <c r="CO6" t="inlineStr">
         <is>
           <t>Neither Agree nor Disagree</t>
@@ -2946,7 +2810,7 @@
       </c>
       <c r="CQ6" t="inlineStr">
         <is>
-          <t>Not at all connected</t>
+          <t>Moderately connected</t>
         </is>
       </c>
     </row>
@@ -2963,21 +2827,21 @@
       </c>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="n">
-        <v>1861</v>
+        <v>6007</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>89mv39j4g4w2tmfn</t>
+          <t>s7dcbjderjk847dh</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>06/18/2025 16:45</t>
+          <t>06/21/2025 17:30</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>qualified,Atlantic_City__New_Jersey,/Quota by US Census Region/Origin Region South,/D Apollo Destination 1/Atlantic_City__New_Jersey,/D Apollo State 1/Louisiana,20250617_14:32_v146,Louisiana,/Unemployed and Retired/MSkJW</t>
+          <t>qualified,/D Apollo Destination 1/Denver__Colorado,Denver__Colorado,/Unemployed and Retired/NILhD,/D Apollo State 1/Connecticut,/Quota by US Census Region/Origin Region Northeast,Connecticut,20250617_14:32_v146</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -2987,19 +2851,19 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="J7" t="n">
-        <v>1967</v>
+        <v>1955</v>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>North Carolina</t>
+          <t>New Jersey</t>
         </is>
       </c>
       <c r="L7" t="n">
-        <v>27127</v>
+        <v>7470</v>
       </c>
       <c r="M7" t="inlineStr">
         <is>
@@ -3009,12 +2873,12 @@
       <c r="N7" t="inlineStr"/>
       <c r="O7" t="inlineStr">
         <is>
-          <t>Large city (urban area)</t>
+          <t>Small town (not near an urban area)</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>Employed (full-time)</t>
+          <t>Retired</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr">
@@ -3042,7 +2906,7 @@
       </c>
       <c r="AB7" t="inlineStr">
         <is>
-          <t>High school graduate</t>
+          <t>Some college</t>
         </is>
       </c>
       <c r="AC7" t="inlineStr">
@@ -3061,7 +2925,7 @@
       </c>
       <c r="AI7" t="inlineStr">
         <is>
-          <t>I prefer not to answer</t>
+          <t>Republican</t>
         </is>
       </c>
       <c r="AJ7" t="inlineStr"/>
@@ -3087,7 +2951,7 @@
       </c>
       <c r="AO7" t="inlineStr">
         <is>
-          <t>Neutral – neither good nor poor</t>
+          <t>Poor</t>
         </is>
       </c>
       <c r="AP7" t="inlineStr">
@@ -3097,150 +2961,152 @@
       </c>
       <c r="AQ7" t="inlineStr">
         <is>
-          <t>Neutral – neither good nor poor</t>
+          <t>Poor</t>
         </is>
       </c>
       <c r="AR7" t="inlineStr">
         <is>
+          <t>Neutral – neither good nor poor</t>
+        </is>
+      </c>
+      <c r="AS7" t="inlineStr">
+        <is>
+          <t>Extremely good</t>
+        </is>
+      </c>
+      <c r="AT7" t="inlineStr">
+        <is>
+          <t>Neutral – neither good nor poor</t>
+        </is>
+      </c>
+      <c r="AU7" t="inlineStr">
+        <is>
           <t>Good</t>
         </is>
       </c>
-      <c r="AS7" t="inlineStr">
-        <is>
-          <t>Neutral – neither good nor poor</t>
-        </is>
-      </c>
-      <c r="AT7" t="inlineStr">
-        <is>
-          <t>Neutral – neither good nor poor</t>
-        </is>
-      </c>
-      <c r="AU7" t="inlineStr">
+      <c r="AV7" t="inlineStr">
+        <is>
+          <t>Neutral – neither good nor poor</t>
+        </is>
+      </c>
+      <c r="AW7" t="inlineStr">
+        <is>
+          <t>Extremely poor</t>
+        </is>
+      </c>
+      <c r="AX7" t="inlineStr">
+        <is>
+          <t>Slightly good</t>
+        </is>
+      </c>
+      <c r="AY7" t="inlineStr">
+        <is>
+          <t>Neutral – neither good nor poor</t>
+        </is>
+      </c>
+      <c r="AZ7" t="inlineStr">
+        <is>
+          <t>Poor</t>
+        </is>
+      </c>
+      <c r="BA7" t="inlineStr">
+        <is>
+          <t>Slightly poor</t>
+        </is>
+      </c>
+      <c r="BB7" t="inlineStr">
+        <is>
+          <t>Neutral – neither good nor poor</t>
+        </is>
+      </c>
+      <c r="BC7" t="inlineStr">
+        <is>
+          <t>Poor</t>
+        </is>
+      </c>
+      <c r="BD7" t="inlineStr">
+        <is>
+          <t>Poor</t>
+        </is>
+      </c>
+      <c r="BE7" t="inlineStr">
+        <is>
+          <t>Neutral – neither good nor poor</t>
+        </is>
+      </c>
+      <c r="BF7" t="inlineStr">
+        <is>
+          <t>Slightly poor</t>
+        </is>
+      </c>
+      <c r="BG7" t="inlineStr">
+        <is>
+          <t>Neutral – neither good nor poor</t>
+        </is>
+      </c>
+      <c r="BH7" t="inlineStr">
+        <is>
+          <t>Neutral – neither good nor poor</t>
+        </is>
+      </c>
+      <c r="BI7" t="inlineStr">
+        <is>
+          <t>Poor</t>
+        </is>
+      </c>
+      <c r="BJ7" t="inlineStr">
         <is>
           <t>Good</t>
         </is>
       </c>
-      <c r="AV7" t="inlineStr">
-        <is>
-          <t>Neutral – neither good nor poor</t>
-        </is>
-      </c>
-      <c r="AW7" t="inlineStr">
-        <is>
-          <t>Slightly good</t>
-        </is>
-      </c>
-      <c r="AX7" t="inlineStr">
-        <is>
-          <t>Neutral – neither good nor poor</t>
-        </is>
-      </c>
-      <c r="AY7" t="inlineStr">
-        <is>
-          <t>Neutral – neither good nor poor</t>
-        </is>
-      </c>
-      <c r="AZ7" t="inlineStr">
-        <is>
-          <t>Slightly good</t>
-        </is>
-      </c>
-      <c r="BA7" t="inlineStr">
-        <is>
-          <t>Neutral – neither good nor poor</t>
-        </is>
-      </c>
-      <c r="BB7" t="inlineStr">
-        <is>
-          <t>Neutral – neither good nor poor</t>
-        </is>
-      </c>
-      <c r="BC7" t="inlineStr">
+      <c r="BK7" t="inlineStr">
+        <is>
+          <t>Neutral – neither good nor poor</t>
+        </is>
+      </c>
+      <c r="BL7" t="inlineStr">
+        <is>
+          <t>Neutral – neither good nor poor</t>
+        </is>
+      </c>
+      <c r="BM7" t="inlineStr">
+        <is>
+          <t>Neutral – neither good nor poor</t>
+        </is>
+      </c>
+      <c r="BN7" t="inlineStr">
         <is>
           <t>Good</t>
         </is>
       </c>
-      <c r="BD7" t="inlineStr">
-        <is>
-          <t>Good</t>
-        </is>
-      </c>
-      <c r="BE7" t="inlineStr">
-        <is>
-          <t>Good</t>
-        </is>
-      </c>
-      <c r="BF7" t="inlineStr">
-        <is>
-          <t>Neutral – neither good nor poor</t>
-        </is>
-      </c>
-      <c r="BG7" t="inlineStr">
-        <is>
-          <t>Neutral – neither good nor poor</t>
-        </is>
-      </c>
-      <c r="BH7" t="inlineStr">
-        <is>
-          <t>Good</t>
-        </is>
-      </c>
-      <c r="BI7" t="inlineStr">
-        <is>
-          <t>Slightly good</t>
-        </is>
-      </c>
-      <c r="BJ7" t="inlineStr">
-        <is>
-          <t>Slightly good</t>
-        </is>
-      </c>
-      <c r="BK7" t="inlineStr">
-        <is>
-          <t>Slightly good</t>
-        </is>
-      </c>
-      <c r="BL7" t="inlineStr">
-        <is>
-          <t>Neutral – neither good nor poor</t>
-        </is>
-      </c>
-      <c r="BM7" t="inlineStr">
-        <is>
-          <t>Neutral – neither good nor poor</t>
-        </is>
-      </c>
-      <c r="BN7" t="inlineStr">
-        <is>
-          <t>Neutral – neither good nor poor</t>
-        </is>
-      </c>
       <c r="BO7" t="inlineStr">
         <is>
-          <t>Extremely unappealing</t>
+          <t>Neutral (neither appealing nor unappealing)</t>
         </is>
       </c>
       <c r="BP7" t="inlineStr">
         <is>
-          <t>Extremely unappealing</t>
+          <t>Neutral (neither appealing nor unappealing)</t>
         </is>
       </c>
       <c r="BQ7" t="inlineStr">
         <is>
-          <t>I don’t know</t>
-        </is>
-      </c>
-      <c r="BR7" t="n">
-        <v>5</v>
+          <t>Unchanged (neither more nor less popular)</t>
+        </is>
+      </c>
+      <c r="BR7" t="inlineStr">
+        <is>
+          <t>0 - NOT AT ALL UNIQUE</t>
+        </is>
       </c>
       <c r="BS7" t="inlineStr">
         <is>
-          <t>Slightly welcoming</t>
+          <t>Neutral (neither welcoming nor unwelcoming)</t>
         </is>
       </c>
       <c r="BT7" t="inlineStr">
         <is>
-          <t>B-</t>
+          <t>C</t>
         </is>
       </c>
       <c r="BU7" t="inlineStr">
@@ -3270,7 +3136,7 @@
       </c>
       <c r="BZ7" t="inlineStr">
         <is>
-          <t>Extremely unappealing</t>
+          <t>Neutral (neither appealing nor unappealing)</t>
         </is>
       </c>
       <c r="CA7" t="inlineStr">
@@ -3290,7 +3156,7 @@
       </c>
       <c r="CD7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>I don’t know enough about the destination</t>
         </is>
       </c>
       <c r="CE7" t="inlineStr">
@@ -3305,7 +3171,7 @@
       </c>
       <c r="CG7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>It’s too expensive</t>
         </is>
       </c>
       <c r="CH7" t="inlineStr">
@@ -3315,7 +3181,7 @@
       </c>
       <c r="CI7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>It’s too far away/too hard to get to</t>
         </is>
       </c>
       <c r="CJ7" t="inlineStr">
@@ -3345,12 +3211,12 @@
       </c>
       <c r="CO7" t="inlineStr">
         <is>
-          <t>Neither Agree nor Disagree</t>
+          <t>Disagree</t>
         </is>
       </c>
       <c r="CP7" t="inlineStr">
         <is>
-          <t>Neither Agree nor Disagree</t>
+          <t>Disagree</t>
         </is>
       </c>
       <c r="CQ7" t="inlineStr">
@@ -3372,21 +3238,21 @@
       </c>
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="n">
-        <v>6602</v>
+        <v>3680</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>vpyqrgreay8g67gq</t>
+          <t>hqbtnjwrth182109</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>06/21/2025 23:05</t>
+          <t>06/21/2025 22:13</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>qualified,/D Apollo Destination 1/San_Diego__California,San_Diego__California,/Quota by US Census Region/Origin Region West,/Unemployed and Retired/cJ2Bp,20250617_14:32_v146,Alabama,/D Apollo State 1/Alabama</t>
+          <t>qualified,/Quota by US Census Region/Origin Region South,/D Apollo Destination 1/Los_Angeles__California,/Unemployed and Retired/cJ2Bp,Los_Angeles__California,Rhode_Island,20250617_14:32_v146,/D Apollo State 1/Rhode_Island</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -3396,23 +3262,23 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="J8" t="n">
-        <v>1967</v>
+        <v>1961</v>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>California</t>
+          <t>North Carolina</t>
         </is>
       </c>
       <c r="L8" t="n">
-        <v>94509</v>
+        <v>27560</v>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>$50,000 to $79,999</t>
+          <t>$30,000 to $49,999</t>
         </is>
       </c>
       <c r="N8" t="inlineStr"/>
@@ -3446,17 +3312,17 @@
       <c r="Z8" t="inlineStr"/>
       <c r="AA8" t="inlineStr">
         <is>
-          <t>Hispanic/Latino</t>
+          <t>Black/African-American</t>
         </is>
       </c>
       <c r="AB8" t="inlineStr">
         <is>
-          <t>Some graduate school</t>
+          <t>Some college</t>
         </is>
       </c>
       <c r="AC8" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Married</t>
         </is>
       </c>
       <c r="AD8" t="inlineStr"/>
@@ -3481,170 +3347,170 @@
       </c>
       <c r="AL8" t="inlineStr">
         <is>
-          <t>Slightly familiar</t>
+          <t>Unfamiliar</t>
         </is>
       </c>
       <c r="AM8" t="inlineStr">
         <is>
-          <t>Neutral (neither likely nor unlikely)</t>
+          <t>Unlikely</t>
         </is>
       </c>
       <c r="AN8" t="inlineStr">
         <is>
+          <t>Slightly good</t>
+        </is>
+      </c>
+      <c r="AO8" t="inlineStr">
+        <is>
+          <t>Slightly poor</t>
+        </is>
+      </c>
+      <c r="AP8" t="inlineStr">
+        <is>
+          <t>Slightly poor</t>
+        </is>
+      </c>
+      <c r="AQ8" t="inlineStr">
+        <is>
+          <t>Neutral – neither good nor poor</t>
+        </is>
+      </c>
+      <c r="AR8" t="inlineStr">
+        <is>
+          <t>Neutral – neither good nor poor</t>
+        </is>
+      </c>
+      <c r="AS8" t="inlineStr">
+        <is>
+          <t>Poor</t>
+        </is>
+      </c>
+      <c r="AT8" t="inlineStr">
+        <is>
+          <t>Slightly good</t>
+        </is>
+      </c>
+      <c r="AU8" t="inlineStr">
+        <is>
+          <t>Neutral – neither good nor poor</t>
+        </is>
+      </c>
+      <c r="AV8" t="inlineStr">
+        <is>
+          <t>Neutral – neither good nor poor</t>
+        </is>
+      </c>
+      <c r="AW8" t="inlineStr">
+        <is>
+          <t>Poor</t>
+        </is>
+      </c>
+      <c r="AX8" t="inlineStr">
+        <is>
+          <t>Neutral – neither good nor poor</t>
+        </is>
+      </c>
+      <c r="AY8" t="inlineStr">
+        <is>
+          <t>Slightly good</t>
+        </is>
+      </c>
+      <c r="AZ8" t="inlineStr">
+        <is>
+          <t>Neutral – neither good nor poor</t>
+        </is>
+      </c>
+      <c r="BA8" t="inlineStr">
+        <is>
+          <t>Slightly poor</t>
+        </is>
+      </c>
+      <c r="BB8" t="inlineStr">
+        <is>
+          <t>Poor</t>
+        </is>
+      </c>
+      <c r="BC8" t="inlineStr">
+        <is>
+          <t>Neutral – neither good nor poor</t>
+        </is>
+      </c>
+      <c r="BD8" t="inlineStr">
+        <is>
+          <t>Slightly good</t>
+        </is>
+      </c>
+      <c r="BE8" t="inlineStr">
+        <is>
+          <t>Slightly poor</t>
+        </is>
+      </c>
+      <c r="BF8" t="inlineStr">
+        <is>
+          <t>Slightly good</t>
+        </is>
+      </c>
+      <c r="BG8" t="inlineStr">
+        <is>
+          <t>Slightly good</t>
+        </is>
+      </c>
+      <c r="BH8" t="inlineStr">
+        <is>
           <t>Good</t>
         </is>
       </c>
-      <c r="AO8" t="inlineStr">
-        <is>
-          <t>Neutral – neither good nor poor</t>
-        </is>
-      </c>
-      <c r="AP8" t="inlineStr">
+      <c r="BI8" t="inlineStr">
+        <is>
+          <t>Slightly poor</t>
+        </is>
+      </c>
+      <c r="BJ8" t="inlineStr">
+        <is>
+          <t>Slightly good</t>
+        </is>
+      </c>
+      <c r="BK8" t="inlineStr">
+        <is>
+          <t>Slightly good</t>
+        </is>
+      </c>
+      <c r="BL8" t="inlineStr">
+        <is>
+          <t>Slightly good</t>
+        </is>
+      </c>
+      <c r="BM8" t="inlineStr">
         <is>
           <t>Good</t>
         </is>
       </c>
-      <c r="AQ8" t="inlineStr">
-        <is>
-          <t>Good</t>
-        </is>
-      </c>
-      <c r="AR8" t="inlineStr">
-        <is>
-          <t>Good</t>
-        </is>
-      </c>
-      <c r="AS8" t="inlineStr">
-        <is>
-          <t>Slightly good</t>
-        </is>
-      </c>
-      <c r="AT8" t="inlineStr">
-        <is>
-          <t>Slightly good</t>
-        </is>
-      </c>
-      <c r="AU8" t="inlineStr">
-        <is>
-          <t>Slightly good</t>
-        </is>
-      </c>
-      <c r="AV8" t="inlineStr">
-        <is>
-          <t>Slightly good</t>
-        </is>
-      </c>
-      <c r="AW8" t="inlineStr">
-        <is>
-          <t>Good</t>
-        </is>
-      </c>
-      <c r="AX8" t="inlineStr">
-        <is>
-          <t>Slightly good</t>
-        </is>
-      </c>
-      <c r="AY8" t="inlineStr">
-        <is>
-          <t>Slightly good</t>
-        </is>
-      </c>
-      <c r="AZ8" t="inlineStr">
-        <is>
-          <t>Neutral – neither good nor poor</t>
-        </is>
-      </c>
-      <c r="BA8" t="inlineStr">
-        <is>
-          <t>Slightly good</t>
-        </is>
-      </c>
-      <c r="BB8" t="inlineStr">
-        <is>
-          <t>Neutral – neither good nor poor</t>
-        </is>
-      </c>
-      <c r="BC8" t="inlineStr">
-        <is>
-          <t>Good</t>
-        </is>
-      </c>
-      <c r="BD8" t="inlineStr">
-        <is>
-          <t>Slightly good</t>
-        </is>
-      </c>
-      <c r="BE8" t="inlineStr">
-        <is>
-          <t>Slightly good</t>
-        </is>
-      </c>
-      <c r="BF8" t="inlineStr">
-        <is>
-          <t>Neutral – neither good nor poor</t>
-        </is>
-      </c>
-      <c r="BG8" t="inlineStr">
-        <is>
-          <t>Slightly good</t>
-        </is>
-      </c>
-      <c r="BH8" t="inlineStr">
-        <is>
-          <t>Good</t>
-        </is>
-      </c>
-      <c r="BI8" t="inlineStr">
-        <is>
-          <t>Slightly good</t>
-        </is>
-      </c>
-      <c r="BJ8" t="inlineStr">
-        <is>
-          <t>Slightly good</t>
-        </is>
-      </c>
-      <c r="BK8" t="inlineStr">
-        <is>
-          <t>Good</t>
-        </is>
-      </c>
-      <c r="BL8" t="inlineStr">
-        <is>
-          <t>Slightly good</t>
-        </is>
-      </c>
-      <c r="BM8" t="inlineStr">
-        <is>
-          <t>Good</t>
-        </is>
-      </c>
       <c r="BN8" t="inlineStr">
         <is>
-          <t>Good</t>
+          <t>Neutral – neither good nor poor</t>
         </is>
       </c>
       <c r="BO8" t="inlineStr">
         <is>
+          <t>Slightly appealing</t>
+        </is>
+      </c>
+      <c r="BP8" t="inlineStr">
+        <is>
           <t>Appealing</t>
         </is>
       </c>
-      <c r="BP8" t="inlineStr">
-        <is>
-          <t>Appealing</t>
-        </is>
-      </c>
       <c r="BQ8" t="inlineStr">
         <is>
-          <t>More popular</t>
+          <t>Unchanged (neither more nor less popular)</t>
         </is>
       </c>
       <c r="BR8" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="BS8" t="inlineStr">
         <is>
-          <t>Welcoming</t>
+          <t>Neutral (neither welcoming nor unwelcoming)</t>
         </is>
       </c>
       <c r="BT8" t="inlineStr">
@@ -3653,26 +3519,26 @@
         </is>
       </c>
       <c r="BU8" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="BV8" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="BW8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="BX8" t="inlineStr">
+        <is>
           <t>No</t>
         </is>
       </c>
-      <c r="BW8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="BX8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
       <c r="BY8" t="inlineStr">
         <is>
-          <t>Agree</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="BZ8" t="inlineStr">
@@ -3683,32 +3549,84 @@
       <c r="CA8" t="n">
         <v>7</v>
       </c>
-      <c r="CB8" t="inlineStr"/>
-      <c r="CC8" t="inlineStr"/>
-      <c r="CD8" t="inlineStr"/>
-      <c r="CE8" t="inlineStr"/>
-      <c r="CF8" t="inlineStr"/>
-      <c r="CG8" t="inlineStr"/>
-      <c r="CH8" t="inlineStr"/>
-      <c r="CI8" t="inlineStr"/>
-      <c r="CJ8" t="inlineStr"/>
-      <c r="CK8" t="inlineStr"/>
-      <c r="CL8" t="inlineStr"/>
-      <c r="CM8" t="inlineStr"/>
-      <c r="CN8" t="inlineStr"/>
+      <c r="CB8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="CC8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="CD8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="CE8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="CF8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="CG8" t="inlineStr">
+        <is>
+          <t>It’s too expensive</t>
+        </is>
+      </c>
+      <c r="CH8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="CI8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="CJ8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="CK8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="CL8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="CM8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="CN8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="CO8" t="inlineStr">
         <is>
-          <t>Agree</t>
+          <t>Disagree</t>
         </is>
       </c>
       <c r="CP8" t="inlineStr">
         <is>
-          <t>Agree</t>
+          <t>Disagree</t>
         </is>
       </c>
       <c r="CQ8" t="inlineStr">
         <is>
-          <t>Slightly connected</t>
+          <t>Moderately connected</t>
         </is>
       </c>
     </row>
@@ -3725,21 +3643,21 @@
       </c>
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="n">
-        <v>6602</v>
+        <v>8760</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>vpyqrgreay8g67gq</t>
+          <t>jxn419t3wxgf43ge</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>06/21/2025 23:05</t>
+          <t>06/22/2025 20:50</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>qualified,/D Apollo Destination 1/San_Diego__California,San_Diego__California,/Quota by US Census Region/Origin Region West,/Unemployed and Retired/cJ2Bp,20250617_14:32_v146,Alabama,/D Apollo State 1/Alabama</t>
+          <t>qualified,/D Apollo Destination 1/Philadelphia__Pennsylvania,20250622_14:03_v148,/D Apollo State 1/Illinois,/Unemployed and Retired/MSkJW,/Quota by US Census Region/Origin Region West,Illinois,Philadelphia__Pennsylvania</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -3753,30 +3671,30 @@
         </is>
       </c>
       <c r="J9" t="n">
-        <v>1967</v>
+        <v>1982</v>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>California</t>
+          <t>Arizona</t>
         </is>
       </c>
       <c r="L9" t="n">
-        <v>94509</v>
+        <v>86440</v>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>$50,000 to $79,999</t>
+          <t>$80,000 to $99,999</t>
         </is>
       </c>
       <c r="N9" t="inlineStr"/>
       <c r="O9" t="inlineStr">
         <is>
-          <t>Suburban area</t>
+          <t>Rural area</t>
         </is>
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>Employed (part-time)</t>
+          <t>Employed (full-time)</t>
         </is>
       </c>
       <c r="Q9" t="inlineStr">
@@ -3786,17 +3704,49 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="S9" t="inlineStr"/>
-      <c r="T9" t="inlineStr"/>
-      <c r="U9" t="inlineStr"/>
-      <c r="V9" t="inlineStr"/>
-      <c r="W9" t="inlineStr"/>
-      <c r="X9" t="inlineStr"/>
-      <c r="Y9" t="inlineStr"/>
-      <c r="Z9" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="W9" t="inlineStr">
+        <is>
+          <t>Psychological issues</t>
+        </is>
+      </c>
+      <c r="X9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Y9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Z9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="AA9" t="inlineStr">
         <is>
           <t>Hispanic/Latino</t>
@@ -3804,12 +3754,12 @@
       </c>
       <c r="AB9" t="inlineStr">
         <is>
-          <t>Some graduate school</t>
+          <t>Completed graduate degree</t>
         </is>
       </c>
       <c r="AC9" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Single</t>
         </is>
       </c>
       <c r="AD9" t="inlineStr"/>
@@ -3823,14 +3773,10 @@
       </c>
       <c r="AI9" t="inlineStr">
         <is>
-          <t>Democratic</t>
-        </is>
-      </c>
-      <c r="AJ9" t="inlineStr">
-        <is>
-          <t>Alabama</t>
-        </is>
-      </c>
+          <t>Libertarian</t>
+        </is>
+      </c>
+      <c r="AJ9" t="inlineStr"/>
       <c r="AK9" t="inlineStr">
         <is>
           <t>Zero</t>
@@ -3848,7 +3794,7 @@
       </c>
       <c r="AN9" t="inlineStr">
         <is>
-          <t>Neutral – neither good nor poor</t>
+          <t>Slightly good</t>
         </is>
       </c>
       <c r="AO9" t="inlineStr">
@@ -3873,12 +3819,12 @@
       </c>
       <c r="AS9" t="inlineStr">
         <is>
-          <t>Neutral – neither good nor poor</t>
+          <t>Slightly good</t>
         </is>
       </c>
       <c r="AT9" t="inlineStr">
         <is>
-          <t>Neutral – neither good nor poor</t>
+          <t>Good</t>
         </is>
       </c>
       <c r="AU9" t="inlineStr">
@@ -3888,12 +3834,12 @@
       </c>
       <c r="AV9" t="inlineStr">
         <is>
-          <t>Neutral – neither good nor poor</t>
+          <t>Good</t>
         </is>
       </c>
       <c r="AW9" t="inlineStr">
         <is>
-          <t>Neutral – neither good nor poor</t>
+          <t>Slightly good</t>
         </is>
       </c>
       <c r="AX9" t="inlineStr">
@@ -3903,12 +3849,12 @@
       </c>
       <c r="AY9" t="inlineStr">
         <is>
-          <t>Neutral – neither good nor poor</t>
+          <t>Slightly good</t>
         </is>
       </c>
       <c r="AZ9" t="inlineStr">
         <is>
-          <t>Neutral – neither good nor poor</t>
+          <t>Good</t>
         </is>
       </c>
       <c r="BA9" t="inlineStr">
@@ -3918,22 +3864,22 @@
       </c>
       <c r="BB9" t="inlineStr">
         <is>
-          <t>Neutral – neither good nor poor</t>
+          <t>Slightly poor</t>
         </is>
       </c>
       <c r="BC9" t="inlineStr">
         <is>
-          <t>Neutral – neither good nor poor</t>
+          <t>Good</t>
         </is>
       </c>
       <c r="BD9" t="inlineStr">
         <is>
-          <t>Neutral – neither good nor poor</t>
+          <t>Good</t>
         </is>
       </c>
       <c r="BE9" t="inlineStr">
         <is>
-          <t>Neutral – neither good nor poor</t>
+          <t>Good</t>
         </is>
       </c>
       <c r="BF9" t="inlineStr">
@@ -3943,52 +3889,52 @@
       </c>
       <c r="BG9" t="inlineStr">
         <is>
-          <t>Neutral – neither good nor poor</t>
+          <t>Good</t>
         </is>
       </c>
       <c r="BH9" t="inlineStr">
         <is>
-          <t>Neutral – neither good nor poor</t>
+          <t>Slightly good</t>
         </is>
       </c>
       <c r="BI9" t="inlineStr">
         <is>
-          <t>Neutral – neither good nor poor</t>
+          <t>Good</t>
         </is>
       </c>
       <c r="BJ9" t="inlineStr">
         <is>
-          <t>Neutral – neither good nor poor</t>
+          <t>Slightly good</t>
         </is>
       </c>
       <c r="BK9" t="inlineStr">
         <is>
-          <t>Neutral – neither good nor poor</t>
+          <t>Good</t>
         </is>
       </c>
       <c r="BL9" t="inlineStr">
         <is>
-          <t>Neutral – neither good nor poor</t>
+          <t>Good</t>
         </is>
       </c>
       <c r="BM9" t="inlineStr">
         <is>
-          <t>Neutral – neither good nor poor</t>
+          <t>Slightly good</t>
         </is>
       </c>
       <c r="BN9" t="inlineStr">
         <is>
-          <t>Neutral – neither good nor poor</t>
+          <t>Slightly good</t>
         </is>
       </c>
       <c r="BO9" t="inlineStr">
         <is>
-          <t>Neutral (neither appealing nor unappealing)</t>
+          <t>Slightly appealing</t>
         </is>
       </c>
       <c r="BP9" t="inlineStr">
         <is>
-          <t>Neutral (neither appealing nor unappealing)</t>
+          <t>Appealing</t>
         </is>
       </c>
       <c r="BQ9" t="inlineStr">
@@ -3997,22 +3943,20 @@
         </is>
       </c>
       <c r="BR9" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="BS9" t="inlineStr">
         <is>
-          <t>Neutral (neither welcoming nor unwelcoming)</t>
+          <t>Very welcoming</t>
         </is>
       </c>
       <c r="BT9" t="inlineStr">
         <is>
-          <t>B-</t>
-        </is>
-      </c>
-      <c r="BU9" t="inlineStr">
-        <is>
-          <t>0 - NOT AT ALL MOTIVATED</t>
-        </is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="BU9" t="n">
+        <v>7</v>
       </c>
       <c r="BV9" t="inlineStr">
         <is>
@@ -4031,18 +3975,16 @@
       </c>
       <c r="BY9" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Strongly agree</t>
         </is>
       </c>
       <c r="BZ9" t="inlineStr">
         <is>
-          <t>Neutral (neither appealing nor unappealing)</t>
-        </is>
-      </c>
-      <c r="CA9" t="inlineStr">
-        <is>
-          <t>5 – Average accessibility</t>
-        </is>
+          <t>Slightly appealing</t>
+        </is>
+      </c>
+      <c r="CA9" t="n">
+        <v>7</v>
       </c>
       <c r="CB9" t="inlineStr">
         <is>
@@ -4081,7 +4023,7 @@
       </c>
       <c r="CI9" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>It’s too far away/too hard to get to</t>
         </is>
       </c>
       <c r="CJ9" t="inlineStr">
@@ -4106,7 +4048,7 @@
       </c>
       <c r="CN9" t="inlineStr">
         <is>
-          <t>NONE OF THESE</t>
+          <t>-</t>
         </is>
       </c>
       <c r="CO9" t="inlineStr">
@@ -4121,7 +4063,7 @@
       </c>
       <c r="CQ9" t="inlineStr">
         <is>
-          <t>Moderately connected</t>
+          <t>Not at all connected</t>
         </is>
       </c>
     </row>
@@ -4138,21 +4080,21 @@
       </c>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="n">
-        <v>9072</v>
+        <v>7181</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>6fkwnqvqaguewt8c</t>
+          <t>05tev9d85zfq9uzd</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>06/23/2025 01:28</t>
+          <t>06/22/2025 07:49</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>qualified,Georgia,20250622_14:03_v148,/D Apollo Destination 1/Nashville__Tennessee,/D Apollo State 1/Georgia,/Unemployed and Retired/cJ2Bp,Nashville__Tennessee,/Quota by US Census Region/Origin Region Midwest</t>
+          <t>qualified,Nevada,/Quota by US Census Region/Origin Region South,/D Apollo State 1/Nevada,/Unemployed and Retired/cJ2Bp,Montreal_Quebec,20250617_14:32_v146,/D Apollo Destination 1/Montreal_Quebec</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -4162,29 +4104,29 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="J10" t="n">
-        <v>1969</v>
+        <v>1954</v>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>Ohio</t>
+          <t>Maryland</t>
         </is>
       </c>
       <c r="L10" t="n">
-        <v>44641</v>
+        <v>21921</v>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>$100,000 to $124,999</t>
+          <t>$150,000 to $199,999</t>
         </is>
       </c>
       <c r="N10" t="inlineStr"/>
       <c r="O10" t="inlineStr">
         <is>
-          <t>Suburban area</t>
+          <t>Small town (not near an urban area)</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
@@ -4212,12 +4154,12 @@
       <c r="Z10" t="inlineStr"/>
       <c r="AA10" t="inlineStr">
         <is>
-          <t>Native Hawaiian/Pacific Islander</t>
+          <t>White</t>
         </is>
       </c>
       <c r="AB10" t="inlineStr">
         <is>
-          <t>High school graduate</t>
+          <t>Some college</t>
         </is>
       </c>
       <c r="AC10" t="inlineStr">
@@ -4236,7 +4178,7 @@
       </c>
       <c r="AI10" t="inlineStr">
         <is>
-          <t>I prefer not to answer</t>
+          <t>Unaffiliated with a political party</t>
         </is>
       </c>
       <c r="AJ10" t="inlineStr"/>
@@ -4247,132 +4189,132 @@
       </c>
       <c r="AL10" t="inlineStr">
         <is>
-          <t>Unfamiliar</t>
+          <t>Slightly familiar</t>
         </is>
       </c>
       <c r="AM10" t="inlineStr">
         <is>
-          <t>Neutral (neither likely nor unlikely)</t>
+          <t>Unlikely</t>
         </is>
       </c>
       <c r="AN10" t="inlineStr">
         <is>
-          <t>Neutral – neither good nor poor</t>
+          <t>Slightly good</t>
         </is>
       </c>
       <c r="AO10" t="inlineStr">
         <is>
-          <t>Neutral – neither good nor poor</t>
+          <t>Slightly good</t>
         </is>
       </c>
       <c r="AP10" t="inlineStr">
         <is>
-          <t>Neutral – neither good nor poor</t>
+          <t>Slightly good</t>
         </is>
       </c>
       <c r="AQ10" t="inlineStr">
         <is>
-          <t>Neutral – neither good nor poor</t>
+          <t>Slightly good</t>
         </is>
       </c>
       <c r="AR10" t="inlineStr">
         <is>
-          <t>Neutral – neither good nor poor</t>
+          <t>Extremely good</t>
         </is>
       </c>
       <c r="AS10" t="inlineStr">
         <is>
-          <t>Neutral – neither good nor poor</t>
+          <t>Slightly good</t>
         </is>
       </c>
       <c r="AT10" t="inlineStr">
         <is>
-          <t>Neutral – neither good nor poor</t>
+          <t>Good</t>
         </is>
       </c>
       <c r="AU10" t="inlineStr">
         <is>
-          <t>Neutral – neither good nor poor</t>
+          <t>Extremely good</t>
         </is>
       </c>
       <c r="AV10" t="inlineStr">
         <is>
-          <t>Neutral – neither good nor poor</t>
+          <t>Slightly good</t>
         </is>
       </c>
       <c r="AW10" t="inlineStr">
         <is>
-          <t>Neutral – neither good nor poor</t>
+          <t>Slightly good</t>
         </is>
       </c>
       <c r="AX10" t="inlineStr">
         <is>
-          <t>Neutral – neither good nor poor</t>
+          <t>Good</t>
         </is>
       </c>
       <c r="AY10" t="inlineStr">
         <is>
-          <t>Neutral – neither good nor poor</t>
+          <t>Good</t>
         </is>
       </c>
       <c r="AZ10" t="inlineStr">
         <is>
-          <t>Neutral – neither good nor poor</t>
+          <t>Good</t>
         </is>
       </c>
       <c r="BA10" t="inlineStr">
         <is>
-          <t>Neutral – neither good nor poor</t>
+          <t>Good</t>
         </is>
       </c>
       <c r="BB10" t="inlineStr">
         <is>
-          <t>Neutral – neither good nor poor</t>
+          <t>Good</t>
         </is>
       </c>
       <c r="BC10" t="inlineStr">
         <is>
-          <t>Neutral – neither good nor poor</t>
+          <t>Extremely good</t>
         </is>
       </c>
       <c r="BD10" t="inlineStr">
         <is>
-          <t>Neutral – neither good nor poor</t>
+          <t>Good</t>
         </is>
       </c>
       <c r="BE10" t="inlineStr">
         <is>
-          <t>Neutral – neither good nor poor</t>
+          <t>Good</t>
         </is>
       </c>
       <c r="BF10" t="inlineStr">
         <is>
-          <t>Neutral – neither good nor poor</t>
+          <t>Good</t>
         </is>
       </c>
       <c r="BG10" t="inlineStr">
         <is>
-          <t>Neutral – neither good nor poor</t>
+          <t>Slightly good</t>
         </is>
       </c>
       <c r="BH10" t="inlineStr">
         <is>
-          <t>Neutral – neither good nor poor</t>
+          <t>Slightly good</t>
         </is>
       </c>
       <c r="BI10" t="inlineStr">
         <is>
-          <t>Neutral – neither good nor poor</t>
+          <t>Extremely good</t>
         </is>
       </c>
       <c r="BJ10" t="inlineStr">
         <is>
-          <t>Neutral – neither good nor poor</t>
+          <t>Slightly good</t>
         </is>
       </c>
       <c r="BK10" t="inlineStr">
         <is>
-          <t>Neutral – neither good nor poor</t>
+          <t>Good</t>
         </is>
       </c>
       <c r="BL10" t="inlineStr">
@@ -4382,44 +4324,44 @@
       </c>
       <c r="BM10" t="inlineStr">
         <is>
-          <t>Neutral – neither good nor poor</t>
+          <t>Slightly good</t>
         </is>
       </c>
       <c r="BN10" t="inlineStr">
         <is>
-          <t>Neutral – neither good nor poor</t>
+          <t>Good</t>
         </is>
       </c>
       <c r="BO10" t="inlineStr">
         <is>
-          <t>Slightly appealing</t>
+          <t>Appealing</t>
         </is>
       </c>
       <c r="BP10" t="inlineStr">
         <is>
-          <t>Neutral (neither appealing nor unappealing)</t>
+          <t>Appealing</t>
         </is>
       </c>
       <c r="BQ10" t="inlineStr">
         <is>
-          <t>I don’t know</t>
+          <t>Unchanged (neither more nor less popular)</t>
         </is>
       </c>
       <c r="BR10" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="BS10" t="inlineStr">
         <is>
-          <t>Neutral (neither welcoming nor unwelcoming)</t>
+          <t>Welcoming</t>
         </is>
       </c>
       <c r="BT10" t="inlineStr">
         <is>
-          <t>A-</t>
+          <t>A</t>
         </is>
       </c>
       <c r="BU10" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="BV10" t="inlineStr">
         <is>
@@ -4438,30 +4380,82 @@
       </c>
       <c r="BY10" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Agree</t>
         </is>
       </c>
       <c r="BZ10" t="inlineStr">
         <is>
-          <t>Neutral (neither appealing nor unappealing)</t>
+          <t>Appealing</t>
         </is>
       </c>
       <c r="CA10" t="n">
         <v>7</v>
       </c>
-      <c r="CB10" t="inlineStr"/>
-      <c r="CC10" t="inlineStr"/>
-      <c r="CD10" t="inlineStr"/>
-      <c r="CE10" t="inlineStr"/>
-      <c r="CF10" t="inlineStr"/>
-      <c r="CG10" t="inlineStr"/>
-      <c r="CH10" t="inlineStr"/>
-      <c r="CI10" t="inlineStr"/>
-      <c r="CJ10" t="inlineStr"/>
-      <c r="CK10" t="inlineStr"/>
-      <c r="CL10" t="inlineStr"/>
-      <c r="CM10" t="inlineStr"/>
-      <c r="CN10" t="inlineStr"/>
+      <c r="CB10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="CC10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="CD10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="CE10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="CF10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="CG10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="CH10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="CI10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="CJ10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="CK10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="CL10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="CM10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="CN10" t="inlineStr">
+        <is>
+          <t>NONE OF THESE</t>
+        </is>
+      </c>
       <c r="CO10" t="inlineStr">
         <is>
           <t>Neither Agree nor Disagree</t>
@@ -4491,21 +4485,21 @@
       </c>
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="n">
-        <v>9072</v>
+        <v>1861</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>6fkwnqvqaguewt8c</t>
+          <t>89mv39j4g4w2tmfn</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>06/23/2025 01:28</t>
+          <t>06/18/2025 16:45</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>qualified,Georgia,20250622_14:03_v148,/D Apollo Destination 1/Nashville__Tennessee,/D Apollo State 1/Georgia,/Unemployed and Retired/cJ2Bp,Nashville__Tennessee,/Quota by US Census Region/Origin Region Midwest</t>
+          <t>qualified,Atlantic_City__New_Jersey,/Quota by US Census Region/Origin Region South,/D Apollo Destination 1/Atlantic_City__New_Jersey,/D Apollo State 1/Louisiana,20250617_14:32_v146,Louisiana,/Unemployed and Retired/MSkJW</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -4519,30 +4513,30 @@
         </is>
       </c>
       <c r="J11" t="n">
-        <v>1969</v>
+        <v>1967</v>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>Ohio</t>
+          <t>North Carolina</t>
         </is>
       </c>
       <c r="L11" t="n">
-        <v>44641</v>
+        <v>27127</v>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>$100,000 to $124,999</t>
+          <t>$30,000 to $49,999</t>
         </is>
       </c>
       <c r="N11" t="inlineStr"/>
       <c r="O11" t="inlineStr">
         <is>
-          <t>Suburban area</t>
+          <t>Large city (urban area)</t>
         </is>
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>Employed (part-time)</t>
+          <t>Employed (full-time)</t>
         </is>
       </c>
       <c r="Q11" t="inlineStr">
@@ -4565,7 +4559,7 @@
       <c r="Z11" t="inlineStr"/>
       <c r="AA11" t="inlineStr">
         <is>
-          <t>Native Hawaiian/Pacific Islander</t>
+          <t>White</t>
         </is>
       </c>
       <c r="AB11" t="inlineStr">
@@ -4593,17 +4587,19 @@
         </is>
       </c>
       <c r="AJ11" t="inlineStr"/>
-      <c r="AK11" t="n">
-        <v>2</v>
+      <c r="AK11" t="inlineStr">
+        <is>
+          <t>Zero</t>
+        </is>
       </c>
       <c r="AL11" t="inlineStr">
         <is>
-          <t>Neutral (neither familiar nor unfamiliar)</t>
+          <t>Totally unfamiliar</t>
         </is>
       </c>
       <c r="AM11" t="inlineStr">
         <is>
-          <t>Neutral (neither likely nor unlikely)</t>
+          <t>Extremely unlikely</t>
         </is>
       </c>
       <c r="AN11" t="inlineStr">
@@ -4628,7 +4624,7 @@
       </c>
       <c r="AR11" t="inlineStr">
         <is>
-          <t>Neutral – neither good nor poor</t>
+          <t>Good</t>
         </is>
       </c>
       <c r="AS11" t="inlineStr">
@@ -4643,7 +4639,7 @@
       </c>
       <c r="AU11" t="inlineStr">
         <is>
-          <t>Neutral – neither good nor poor</t>
+          <t>Good</t>
         </is>
       </c>
       <c r="AV11" t="inlineStr">
@@ -4653,7 +4649,7 @@
       </c>
       <c r="AW11" t="inlineStr">
         <is>
-          <t>Neutral – neither good nor poor</t>
+          <t>Slightly good</t>
         </is>
       </c>
       <c r="AX11" t="inlineStr">
@@ -4668,7 +4664,7 @@
       </c>
       <c r="AZ11" t="inlineStr">
         <is>
-          <t>Neutral – neither good nor poor</t>
+          <t>Slightly good</t>
         </is>
       </c>
       <c r="BA11" t="inlineStr">
@@ -4683,17 +4679,17 @@
       </c>
       <c r="BC11" t="inlineStr">
         <is>
-          <t>Neutral – neither good nor poor</t>
+          <t>Good</t>
         </is>
       </c>
       <c r="BD11" t="inlineStr">
         <is>
-          <t>Neutral – neither good nor poor</t>
+          <t>Good</t>
         </is>
       </c>
       <c r="BE11" t="inlineStr">
         <is>
-          <t>Neutral – neither good nor poor</t>
+          <t>Good</t>
         </is>
       </c>
       <c r="BF11" t="inlineStr">
@@ -4708,22 +4704,22 @@
       </c>
       <c r="BH11" t="inlineStr">
         <is>
-          <t>Neutral – neither good nor poor</t>
+          <t>Good</t>
         </is>
       </c>
       <c r="BI11" t="inlineStr">
         <is>
-          <t>Neutral – neither good nor poor</t>
+          <t>Slightly good</t>
         </is>
       </c>
       <c r="BJ11" t="inlineStr">
         <is>
-          <t>Neutral – neither good nor poor</t>
+          <t>Slightly good</t>
         </is>
       </c>
       <c r="BK11" t="inlineStr">
         <is>
-          <t>Neutral – neither good nor poor</t>
+          <t>Slightly good</t>
         </is>
       </c>
       <c r="BL11" t="inlineStr">
@@ -4743,12 +4739,12 @@
       </c>
       <c r="BO11" t="inlineStr">
         <is>
-          <t>Neutral (neither appealing nor unappealing)</t>
+          <t>Extremely unappealing</t>
         </is>
       </c>
       <c r="BP11" t="inlineStr">
         <is>
-          <t>Neutral (neither appealing nor unappealing)</t>
+          <t>Extremely unappealing</t>
         </is>
       </c>
       <c r="BQ11" t="inlineStr">
@@ -4761,7 +4757,7 @@
       </c>
       <c r="BS11" t="inlineStr">
         <is>
-          <t>Neutral (neither welcoming nor unwelcoming)</t>
+          <t>Slightly welcoming</t>
         </is>
       </c>
       <c r="BT11" t="inlineStr">
@@ -4769,22 +4765,24 @@
           <t>B-</t>
         </is>
       </c>
-      <c r="BU11" t="n">
-        <v>4</v>
+      <c r="BU11" t="inlineStr">
+        <is>
+          <t>0 - NOT AT ALL MOTIVATED</t>
+        </is>
       </c>
       <c r="BV11" t="inlineStr">
         <is>
-          <t>I don’t know</t>
+          <t>No</t>
         </is>
       </c>
       <c r="BW11" t="inlineStr">
         <is>
-          <t>I don’t know</t>
+          <t>No</t>
         </is>
       </c>
       <c r="BX11" t="inlineStr">
         <is>
-          <t>I don’t know</t>
+          <t>No</t>
         </is>
       </c>
       <c r="BY11" t="inlineStr">
@@ -4794,7 +4792,7 @@
       </c>
       <c r="BZ11" t="inlineStr">
         <is>
-          <t>Neutral (neither appealing nor unappealing)</t>
+          <t>Extremely unappealing</t>
         </is>
       </c>
       <c r="CA11" t="inlineStr">
@@ -4802,19 +4800,71 @@
           <t>5 – Average accessibility</t>
         </is>
       </c>
-      <c r="CB11" t="inlineStr"/>
-      <c r="CC11" t="inlineStr"/>
-      <c r="CD11" t="inlineStr"/>
-      <c r="CE11" t="inlineStr"/>
-      <c r="CF11" t="inlineStr"/>
-      <c r="CG11" t="inlineStr"/>
-      <c r="CH11" t="inlineStr"/>
-      <c r="CI11" t="inlineStr"/>
-      <c r="CJ11" t="inlineStr"/>
-      <c r="CK11" t="inlineStr"/>
-      <c r="CL11" t="inlineStr"/>
-      <c r="CM11" t="inlineStr"/>
-      <c r="CN11" t="inlineStr"/>
+      <c r="CB11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="CC11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="CD11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="CE11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="CF11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="CG11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="CH11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="CI11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="CJ11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="CK11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="CL11" t="inlineStr">
+        <is>
+          <t>The destination is just not on my radar</t>
+        </is>
+      </c>
+      <c r="CM11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="CN11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="CO11" t="inlineStr">
         <is>
           <t>Neither Agree nor Disagree</t>
@@ -4827,7 +4877,7 @@
       </c>
       <c r="CQ11" t="inlineStr">
         <is>
-          <t>Moderately connected</t>
+          <t>Not at all connected</t>
         </is>
       </c>
     </row>
@@ -4844,21 +4894,21 @@
       </c>
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="n">
-        <v>6007</v>
+        <v>6602</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>s7dcbjderjk847dh</t>
+          <t>vpyqrgreay8g67gq</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>06/21/2025 17:30</t>
+          <t>06/21/2025 23:05</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>qualified,/D Apollo Destination 1/Denver__Colorado,Denver__Colorado,/Unemployed and Retired/NILhD,/D Apollo State 1/Connecticut,/Quota by US Census Region/Origin Region Northeast,Connecticut,20250617_14:32_v146</t>
+          <t>qualified,/D Apollo Destination 1/San_Diego__California,San_Diego__California,/Quota by US Census Region/Origin Region West,/Unemployed and Retired/cJ2Bp,20250617_14:32_v146,Alabama,/D Apollo State 1/Alabama</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -4868,34 +4918,34 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="J12" t="n">
-        <v>1955</v>
+        <v>1967</v>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>New Jersey</t>
+          <t>California</t>
         </is>
       </c>
       <c r="L12" t="n">
-        <v>7470</v>
+        <v>94509</v>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>$30,000 to $49,999</t>
+          <t>$50,000 to $79,999</t>
         </is>
       </c>
       <c r="N12" t="inlineStr"/>
       <c r="O12" t="inlineStr">
         <is>
-          <t>Small town (not near an urban area)</t>
+          <t>Suburban area</t>
         </is>
       </c>
       <c r="P12" t="inlineStr">
         <is>
-          <t>Retired</t>
+          <t>Employed (part-time)</t>
         </is>
       </c>
       <c r="Q12" t="inlineStr">
@@ -4918,17 +4968,17 @@
       <c r="Z12" t="inlineStr"/>
       <c r="AA12" t="inlineStr">
         <is>
-          <t>White</t>
+          <t>Hispanic/Latino</t>
         </is>
       </c>
       <c r="AB12" t="inlineStr">
         <is>
-          <t>Some college</t>
+          <t>Some graduate school</t>
         </is>
       </c>
       <c r="AC12" t="inlineStr">
         <is>
-          <t>Married</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="AD12" t="inlineStr"/>
@@ -4942,10 +4992,14 @@
       </c>
       <c r="AI12" t="inlineStr">
         <is>
-          <t>Republican</t>
-        </is>
-      </c>
-      <c r="AJ12" t="inlineStr"/>
+          <t>Democratic</t>
+        </is>
+      </c>
+      <c r="AJ12" t="inlineStr">
+        <is>
+          <t>Alabama</t>
+        </is>
+      </c>
       <c r="AK12" t="inlineStr">
         <is>
           <t>Zero</t>
@@ -4953,12 +5007,12 @@
       </c>
       <c r="AL12" t="inlineStr">
         <is>
-          <t>Totally unfamiliar</t>
+          <t>Unfamiliar</t>
         </is>
       </c>
       <c r="AM12" t="inlineStr">
         <is>
-          <t>Extremely unlikely</t>
+          <t>Unlikely</t>
         </is>
       </c>
       <c r="AN12" t="inlineStr">
@@ -4968,7 +5022,7 @@
       </c>
       <c r="AO12" t="inlineStr">
         <is>
-          <t>Poor</t>
+          <t>Neutral – neither good nor poor</t>
         </is>
       </c>
       <c r="AP12" t="inlineStr">
@@ -4978,7 +5032,7 @@
       </c>
       <c r="AQ12" t="inlineStr">
         <is>
-          <t>Poor</t>
+          <t>Neutral – neither good nor poor</t>
         </is>
       </c>
       <c r="AR12" t="inlineStr">
@@ -4988,7 +5042,7 @@
       </c>
       <c r="AS12" t="inlineStr">
         <is>
-          <t>Extremely good</t>
+          <t>Neutral – neither good nor poor</t>
         </is>
       </c>
       <c r="AT12" t="inlineStr">
@@ -4998,7 +5052,7 @@
       </c>
       <c r="AU12" t="inlineStr">
         <is>
-          <t>Good</t>
+          <t>Neutral – neither good nor poor</t>
         </is>
       </c>
       <c r="AV12" t="inlineStr">
@@ -5008,12 +5062,12 @@
       </c>
       <c r="AW12" t="inlineStr">
         <is>
-          <t>Extremely poor</t>
+          <t>Neutral – neither good nor poor</t>
         </is>
       </c>
       <c r="AX12" t="inlineStr">
         <is>
-          <t>Slightly good</t>
+          <t>Neutral – neither good nor poor</t>
         </is>
       </c>
       <c r="AY12" t="inlineStr">
@@ -5023,12 +5077,12 @@
       </c>
       <c r="AZ12" t="inlineStr">
         <is>
-          <t>Poor</t>
+          <t>Neutral – neither good nor poor</t>
         </is>
       </c>
       <c r="BA12" t="inlineStr">
         <is>
-          <t>Slightly poor</t>
+          <t>Neutral – neither good nor poor</t>
         </is>
       </c>
       <c r="BB12" t="inlineStr">
@@ -5038,12 +5092,12 @@
       </c>
       <c r="BC12" t="inlineStr">
         <is>
-          <t>Poor</t>
+          <t>Neutral – neither good nor poor</t>
         </is>
       </c>
       <c r="BD12" t="inlineStr">
         <is>
-          <t>Poor</t>
+          <t>Neutral – neither good nor poor</t>
         </is>
       </c>
       <c r="BE12" t="inlineStr">
@@ -5053,7 +5107,7 @@
       </c>
       <c r="BF12" t="inlineStr">
         <is>
-          <t>Slightly poor</t>
+          <t>Neutral – neither good nor poor</t>
         </is>
       </c>
       <c r="BG12" t="inlineStr">
@@ -5068,12 +5122,12 @@
       </c>
       <c r="BI12" t="inlineStr">
         <is>
-          <t>Poor</t>
+          <t>Neutral – neither good nor poor</t>
         </is>
       </c>
       <c r="BJ12" t="inlineStr">
         <is>
-          <t>Good</t>
+          <t>Neutral – neither good nor poor</t>
         </is>
       </c>
       <c r="BK12" t="inlineStr">
@@ -5093,7 +5147,7 @@
       </c>
       <c r="BN12" t="inlineStr">
         <is>
-          <t>Good</t>
+          <t>Neutral – neither good nor poor</t>
         </is>
       </c>
       <c r="BO12" t="inlineStr">
@@ -5111,10 +5165,8 @@
           <t>Unchanged (neither more nor less popular)</t>
         </is>
       </c>
-      <c r="BR12" t="inlineStr">
-        <is>
-          <t>0 - NOT AT ALL UNIQUE</t>
-        </is>
+      <c r="BR12" t="n">
+        <v>5</v>
       </c>
       <c r="BS12" t="inlineStr">
         <is>
@@ -5123,7 +5175,7 @@
       </c>
       <c r="BT12" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B-</t>
         </is>
       </c>
       <c r="BU12" t="inlineStr">
@@ -5173,7 +5225,7 @@
       </c>
       <c r="CD12" t="inlineStr">
         <is>
-          <t>I don’t know enough about the destination</t>
+          <t>-</t>
         </is>
       </c>
       <c r="CE12" t="inlineStr">
@@ -5188,7 +5240,7 @@
       </c>
       <c r="CG12" t="inlineStr">
         <is>
-          <t>It’s too expensive</t>
+          <t>-</t>
         </is>
       </c>
       <c r="CH12" t="inlineStr">
@@ -5198,7 +5250,7 @@
       </c>
       <c r="CI12" t="inlineStr">
         <is>
-          <t>It’s too far away/too hard to get to</t>
+          <t>-</t>
         </is>
       </c>
       <c r="CJ12" t="inlineStr">
@@ -5213,7 +5265,7 @@
       </c>
       <c r="CL12" t="inlineStr">
         <is>
-          <t>The destination is just not on my radar</t>
+          <t>-</t>
         </is>
       </c>
       <c r="CM12" t="inlineStr">
@@ -5223,22 +5275,22 @@
       </c>
       <c r="CN12" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>NONE OF THESE</t>
         </is>
       </c>
       <c r="CO12" t="inlineStr">
         <is>
-          <t>Disagree</t>
+          <t>Neither Agree nor Disagree</t>
         </is>
       </c>
       <c r="CP12" t="inlineStr">
         <is>
-          <t>Disagree</t>
+          <t>Neither Agree nor Disagree</t>
         </is>
       </c>
       <c r="CQ12" t="inlineStr">
         <is>
-          <t>Not at all connected</t>
+          <t>Moderately connected</t>
         </is>
       </c>
     </row>
@@ -5255,21 +5307,21 @@
       </c>
       <c r="C13" t="inlineStr"/>
       <c r="D13" t="n">
-        <v>6007</v>
+        <v>9072</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>s7dcbjderjk847dh</t>
+          <t>6fkwnqvqaguewt8c</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>06/21/2025 17:30</t>
+          <t>06/23/2025 01:28</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>qualified,/D Apollo Destination 1/Denver__Colorado,Denver__Colorado,/Unemployed and Retired/NILhD,/D Apollo State 1/Connecticut,/Quota by US Census Region/Origin Region Northeast,Connecticut,20250617_14:32_v146</t>
+          <t>qualified,Georgia,20250622_14:03_v148,/D Apollo Destination 1/Nashville__Tennessee,/D Apollo State 1/Georgia,/Unemployed and Retired/cJ2Bp,Nashville__Tennessee,/Quota by US Census Region/Origin Region Midwest</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -5279,34 +5331,34 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="J13" t="n">
-        <v>1955</v>
+        <v>1969</v>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>New Jersey</t>
+          <t>Ohio</t>
         </is>
       </c>
       <c r="L13" t="n">
-        <v>7470</v>
+        <v>44641</v>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>$30,000 to $49,999</t>
+          <t>$100,000 to $124,999</t>
         </is>
       </c>
       <c r="N13" t="inlineStr"/>
       <c r="O13" t="inlineStr">
         <is>
-          <t>Small town (not near an urban area)</t>
+          <t>Suburban area</t>
         </is>
       </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t>Retired</t>
+          <t>Employed (part-time)</t>
         </is>
       </c>
       <c r="Q13" t="inlineStr">
@@ -5329,12 +5381,12 @@
       <c r="Z13" t="inlineStr"/>
       <c r="AA13" t="inlineStr">
         <is>
-          <t>White</t>
+          <t>Native Hawaiian/Pacific Islander</t>
         </is>
       </c>
       <c r="AB13" t="inlineStr">
         <is>
-          <t>Some college</t>
+          <t>High school graduate</t>
         </is>
       </c>
       <c r="AC13" t="inlineStr">
@@ -5353,168 +5405,166 @@
       </c>
       <c r="AI13" t="inlineStr">
         <is>
-          <t>Republican</t>
+          <t>I prefer not to answer</t>
         </is>
       </c>
       <c r="AJ13" t="inlineStr"/>
-      <c r="AK13" t="inlineStr">
-        <is>
-          <t>Zero</t>
-        </is>
+      <c r="AK13" t="n">
+        <v>2</v>
       </c>
       <c r="AL13" t="inlineStr">
         <is>
-          <t>Totally unfamiliar</t>
+          <t>Neutral (neither familiar nor unfamiliar)</t>
         </is>
       </c>
       <c r="AM13" t="inlineStr">
         <is>
-          <t>Extremely unlikely</t>
+          <t>Neutral (neither likely nor unlikely)</t>
         </is>
       </c>
       <c r="AN13" t="inlineStr">
         <is>
-          <t>Poor</t>
+          <t>Neutral – neither good nor poor</t>
         </is>
       </c>
       <c r="AO13" t="inlineStr">
         <is>
-          <t>Extremely poor</t>
+          <t>Neutral – neither good nor poor</t>
         </is>
       </c>
       <c r="AP13" t="inlineStr">
         <is>
-          <t>Extremely poor</t>
+          <t>Neutral – neither good nor poor</t>
         </is>
       </c>
       <c r="AQ13" t="inlineStr">
         <is>
-          <t>Poor</t>
+          <t>Neutral – neither good nor poor</t>
         </is>
       </c>
       <c r="AR13" t="inlineStr">
         <is>
-          <t>Poor</t>
+          <t>Neutral – neither good nor poor</t>
         </is>
       </c>
       <c r="AS13" t="inlineStr">
         <is>
-          <t>Poor</t>
+          <t>Neutral – neither good nor poor</t>
         </is>
       </c>
       <c r="AT13" t="inlineStr">
         <is>
-          <t>Poor</t>
+          <t>Neutral – neither good nor poor</t>
         </is>
       </c>
       <c r="AU13" t="inlineStr">
         <is>
-          <t>Poor</t>
+          <t>Neutral – neither good nor poor</t>
         </is>
       </c>
       <c r="AV13" t="inlineStr">
         <is>
-          <t>Poor</t>
+          <t>Neutral – neither good nor poor</t>
         </is>
       </c>
       <c r="AW13" t="inlineStr">
         <is>
-          <t>Poor</t>
+          <t>Neutral – neither good nor poor</t>
         </is>
       </c>
       <c r="AX13" t="inlineStr">
         <is>
-          <t>Poor</t>
+          <t>Neutral – neither good nor poor</t>
         </is>
       </c>
       <c r="AY13" t="inlineStr">
         <is>
-          <t>Poor</t>
+          <t>Neutral – neither good nor poor</t>
         </is>
       </c>
       <c r="AZ13" t="inlineStr">
         <is>
-          <t>Poor</t>
+          <t>Neutral – neither good nor poor</t>
         </is>
       </c>
       <c r="BA13" t="inlineStr">
         <is>
-          <t>Poor</t>
+          <t>Neutral – neither good nor poor</t>
         </is>
       </c>
       <c r="BB13" t="inlineStr">
         <is>
-          <t>Extremely poor</t>
+          <t>Neutral – neither good nor poor</t>
         </is>
       </c>
       <c r="BC13" t="inlineStr">
         <is>
-          <t>Poor</t>
+          <t>Neutral – neither good nor poor</t>
         </is>
       </c>
       <c r="BD13" t="inlineStr">
         <is>
-          <t>Poor</t>
+          <t>Neutral – neither good nor poor</t>
         </is>
       </c>
       <c r="BE13" t="inlineStr">
         <is>
-          <t>Poor</t>
+          <t>Neutral – neither good nor poor</t>
         </is>
       </c>
       <c r="BF13" t="inlineStr">
         <is>
-          <t>Poor</t>
+          <t>Neutral – neither good nor poor</t>
         </is>
       </c>
       <c r="BG13" t="inlineStr">
         <is>
-          <t>Poor</t>
+          <t>Neutral – neither good nor poor</t>
         </is>
       </c>
       <c r="BH13" t="inlineStr">
         <is>
-          <t>Extremely poor</t>
+          <t>Neutral – neither good nor poor</t>
         </is>
       </c>
       <c r="BI13" t="inlineStr">
         <is>
-          <t>Extremely poor</t>
+          <t>Neutral – neither good nor poor</t>
         </is>
       </c>
       <c r="BJ13" t="inlineStr">
         <is>
-          <t>Extremely poor</t>
+          <t>Neutral – neither good nor poor</t>
         </is>
       </c>
       <c r="BK13" t="inlineStr">
         <is>
-          <t>Poor</t>
+          <t>Neutral – neither good nor poor</t>
         </is>
       </c>
       <c r="BL13" t="inlineStr">
         <is>
-          <t>Poor</t>
+          <t>Neutral – neither good nor poor</t>
         </is>
       </c>
       <c r="BM13" t="inlineStr">
         <is>
-          <t>Poor</t>
+          <t>Neutral – neither good nor poor</t>
         </is>
       </c>
       <c r="BN13" t="inlineStr">
         <is>
-          <t>Poor</t>
+          <t>Neutral – neither good nor poor</t>
         </is>
       </c>
       <c r="BO13" t="inlineStr">
         <is>
-          <t>Unappealing</t>
+          <t>Neutral (neither appealing nor unappealing)</t>
         </is>
       </c>
       <c r="BP13" t="inlineStr">
         <is>
-          <t>Unappealing</t>
+          <t>Neutral (neither appealing nor unappealing)</t>
         </is>
       </c>
       <c r="BQ13" t="inlineStr">
@@ -5523,34 +5573,34 @@
         </is>
       </c>
       <c r="BR13" t="n">
+        <v>5</v>
+      </c>
+      <c r="BS13" t="inlineStr">
+        <is>
+          <t>Neutral (neither welcoming nor unwelcoming)</t>
+        </is>
+      </c>
+      <c r="BT13" t="inlineStr">
+        <is>
+          <t>B-</t>
+        </is>
+      </c>
+      <c r="BU13" t="n">
         <v>4</v>
       </c>
-      <c r="BS13" t="inlineStr">
-        <is>
-          <t>Neutral (neither welcoming nor unwelcoming)</t>
-        </is>
-      </c>
-      <c r="BT13" t="inlineStr">
-        <is>
-          <t>C+</t>
-        </is>
-      </c>
-      <c r="BU13" t="n">
-        <v>2</v>
-      </c>
       <c r="BV13" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>I don’t know</t>
         </is>
       </c>
       <c r="BW13" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>I don’t know</t>
         </is>
       </c>
       <c r="BX13" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>I don’t know</t>
         </is>
       </c>
       <c r="BY13" t="inlineStr">
@@ -5560,7 +5610,7 @@
       </c>
       <c r="BZ13" t="inlineStr">
         <is>
-          <t>Unappealing</t>
+          <t>Neutral (neither appealing nor unappealing)</t>
         </is>
       </c>
       <c r="CA13" t="inlineStr">
@@ -5568,84 +5618,32 @@
           <t>5 – Average accessibility</t>
         </is>
       </c>
-      <c r="CB13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="CC13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="CD13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="CE13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="CF13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="CG13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="CH13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="CI13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="CJ13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="CK13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="CL13" t="inlineStr">
-        <is>
-          <t>The destination is just not on my radar</t>
-        </is>
-      </c>
-      <c r="CM13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="CN13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+      <c r="CB13" t="inlineStr"/>
+      <c r="CC13" t="inlineStr"/>
+      <c r="CD13" t="inlineStr"/>
+      <c r="CE13" t="inlineStr"/>
+      <c r="CF13" t="inlineStr"/>
+      <c r="CG13" t="inlineStr"/>
+      <c r="CH13" t="inlineStr"/>
+      <c r="CI13" t="inlineStr"/>
+      <c r="CJ13" t="inlineStr"/>
+      <c r="CK13" t="inlineStr"/>
+      <c r="CL13" t="inlineStr"/>
+      <c r="CM13" t="inlineStr"/>
+      <c r="CN13" t="inlineStr"/>
       <c r="CO13" t="inlineStr">
         <is>
-          <t>Disagree</t>
+          <t>Neither Agree nor Disagree</t>
         </is>
       </c>
       <c r="CP13" t="inlineStr">
         <is>
-          <t>Disagree</t>
+          <t>Neither Agree nor Disagree</t>
         </is>
       </c>
       <c r="CQ13" t="inlineStr">
         <is>
-          <t>Not at all connected</t>
+          <t>Moderately connected</t>
         </is>
       </c>
     </row>
@@ -5662,21 +5660,21 @@
       </c>
       <c r="C14" t="inlineStr"/>
       <c r="D14" t="n">
-        <v>3680</v>
+        <v>6007</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>hqbtnjwrth182109</t>
+          <t>s7dcbjderjk847dh</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>06/21/2025 22:13</t>
+          <t>06/21/2025 17:30</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>qualified,/Quota by US Census Region/Origin Region South,/D Apollo Destination 1/Los_Angeles__California,/Unemployed and Retired/cJ2Bp,Los_Angeles__California,Rhode_Island,20250617_14:32_v146,/D Apollo State 1/Rhode_Island</t>
+          <t>qualified,/D Apollo Destination 1/Denver__Colorado,Denver__Colorado,/Unemployed and Retired/NILhD,/D Apollo State 1/Connecticut,/Quota by US Census Region/Origin Region Northeast,Connecticut,20250617_14:32_v146</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -5690,15 +5688,15 @@
         </is>
       </c>
       <c r="J14" t="n">
-        <v>1961</v>
+        <v>1955</v>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>North Carolina</t>
+          <t>New Jersey</t>
         </is>
       </c>
       <c r="L14" t="n">
-        <v>27560</v>
+        <v>7470</v>
       </c>
       <c r="M14" t="inlineStr">
         <is>
@@ -5708,12 +5706,12 @@
       <c r="N14" t="inlineStr"/>
       <c r="O14" t="inlineStr">
         <is>
-          <t>Suburban area</t>
+          <t>Small town (not near an urban area)</t>
         </is>
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>Employed (part-time)</t>
+          <t>Retired</t>
         </is>
       </c>
       <c r="Q14" t="inlineStr">
@@ -5736,7 +5734,7 @@
       <c r="Z14" t="inlineStr"/>
       <c r="AA14" t="inlineStr">
         <is>
-          <t>Black/African-American</t>
+          <t>White</t>
         </is>
       </c>
       <c r="AB14" t="inlineStr">
@@ -5760,7 +5758,7 @@
       </c>
       <c r="AI14" t="inlineStr">
         <is>
-          <t>Democratic</t>
+          <t>Republican</t>
         </is>
       </c>
       <c r="AJ14" t="inlineStr"/>
@@ -5771,37 +5769,37 @@
       </c>
       <c r="AL14" t="inlineStr">
         <is>
-          <t>Unfamiliar</t>
+          <t>Totally unfamiliar</t>
         </is>
       </c>
       <c r="AM14" t="inlineStr">
         <is>
-          <t>Unlikely</t>
+          <t>Extremely unlikely</t>
         </is>
       </c>
       <c r="AN14" t="inlineStr">
         <is>
-          <t>Slightly good</t>
+          <t>Poor</t>
         </is>
       </c>
       <c r="AO14" t="inlineStr">
         <is>
-          <t>Slightly poor</t>
+          <t>Extremely poor</t>
         </is>
       </c>
       <c r="AP14" t="inlineStr">
         <is>
-          <t>Slightly poor</t>
+          <t>Extremely poor</t>
         </is>
       </c>
       <c r="AQ14" t="inlineStr">
         <is>
-          <t>Neutral – neither good nor poor</t>
+          <t>Poor</t>
         </is>
       </c>
       <c r="AR14" t="inlineStr">
         <is>
-          <t>Neutral – neither good nor poor</t>
+          <t>Poor</t>
         </is>
       </c>
       <c r="AS14" t="inlineStr">
@@ -5811,17 +5809,17 @@
       </c>
       <c r="AT14" t="inlineStr">
         <is>
-          <t>Slightly good</t>
+          <t>Poor</t>
         </is>
       </c>
       <c r="AU14" t="inlineStr">
         <is>
-          <t>Neutral – neither good nor poor</t>
+          <t>Poor</t>
         </is>
       </c>
       <c r="AV14" t="inlineStr">
         <is>
-          <t>Neutral – neither good nor poor</t>
+          <t>Poor</t>
         </is>
       </c>
       <c r="AW14" t="inlineStr">
@@ -5831,106 +5829,106 @@
       </c>
       <c r="AX14" t="inlineStr">
         <is>
-          <t>Neutral – neither good nor poor</t>
+          <t>Poor</t>
         </is>
       </c>
       <c r="AY14" t="inlineStr">
         <is>
-          <t>Slightly good</t>
+          <t>Poor</t>
         </is>
       </c>
       <c r="AZ14" t="inlineStr">
         <is>
-          <t>Neutral – neither good nor poor</t>
+          <t>Poor</t>
         </is>
       </c>
       <c r="BA14" t="inlineStr">
         <is>
-          <t>Slightly poor</t>
+          <t>Poor</t>
         </is>
       </c>
       <c r="BB14" t="inlineStr">
         <is>
+          <t>Extremely poor</t>
+        </is>
+      </c>
+      <c r="BC14" t="inlineStr">
+        <is>
           <t>Poor</t>
         </is>
       </c>
-      <c r="BC14" t="inlineStr">
-        <is>
-          <t>Neutral – neither good nor poor</t>
-        </is>
-      </c>
       <c r="BD14" t="inlineStr">
         <is>
-          <t>Slightly good</t>
+          <t>Poor</t>
         </is>
       </c>
       <c r="BE14" t="inlineStr">
         <is>
-          <t>Slightly poor</t>
+          <t>Poor</t>
         </is>
       </c>
       <c r="BF14" t="inlineStr">
         <is>
-          <t>Slightly good</t>
+          <t>Poor</t>
         </is>
       </c>
       <c r="BG14" t="inlineStr">
         <is>
-          <t>Slightly good</t>
+          <t>Poor</t>
         </is>
       </c>
       <c r="BH14" t="inlineStr">
         <is>
-          <t>Good</t>
+          <t>Extremely poor</t>
         </is>
       </c>
       <c r="BI14" t="inlineStr">
         <is>
-          <t>Slightly poor</t>
+          <t>Extremely poor</t>
         </is>
       </c>
       <c r="BJ14" t="inlineStr">
         <is>
-          <t>Slightly good</t>
+          <t>Extremely poor</t>
         </is>
       </c>
       <c r="BK14" t="inlineStr">
         <is>
-          <t>Slightly good</t>
+          <t>Poor</t>
         </is>
       </c>
       <c r="BL14" t="inlineStr">
         <is>
-          <t>Slightly good</t>
+          <t>Poor</t>
         </is>
       </c>
       <c r="BM14" t="inlineStr">
         <is>
-          <t>Good</t>
+          <t>Poor</t>
         </is>
       </c>
       <c r="BN14" t="inlineStr">
         <is>
-          <t>Neutral – neither good nor poor</t>
+          <t>Poor</t>
         </is>
       </c>
       <c r="BO14" t="inlineStr">
         <is>
-          <t>Slightly appealing</t>
+          <t>Unappealing</t>
         </is>
       </c>
       <c r="BP14" t="inlineStr">
         <is>
-          <t>Appealing</t>
+          <t>Unappealing</t>
         </is>
       </c>
       <c r="BQ14" t="inlineStr">
         <is>
-          <t>Unchanged (neither more nor less popular)</t>
+          <t>I don’t know</t>
         </is>
       </c>
       <c r="BR14" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="BS14" t="inlineStr">
         <is>
@@ -5939,7 +5937,7 @@
       </c>
       <c r="BT14" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C+</t>
         </is>
       </c>
       <c r="BU14" t="n">
@@ -5947,12 +5945,12 @@
       </c>
       <c r="BV14" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="BW14" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="BX14" t="inlineStr">
@@ -5967,11 +5965,13 @@
       </c>
       <c r="BZ14" t="inlineStr">
         <is>
-          <t>Slightly appealing</t>
-        </is>
-      </c>
-      <c r="CA14" t="n">
-        <v>7</v>
+          <t>Unappealing</t>
+        </is>
+      </c>
+      <c r="CA14" t="inlineStr">
+        <is>
+          <t>5 – Average accessibility</t>
+        </is>
       </c>
       <c r="CB14" t="inlineStr">
         <is>
@@ -6000,7 +6000,7 @@
       </c>
       <c r="CG14" t="inlineStr">
         <is>
-          <t>It’s too expensive</t>
+          <t>-</t>
         </is>
       </c>
       <c r="CH14" t="inlineStr">
@@ -6025,7 +6025,7 @@
       </c>
       <c r="CL14" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>The destination is just not on my radar</t>
         </is>
       </c>
       <c r="CM14" t="inlineStr">
@@ -6050,7 +6050,7 @@
       </c>
       <c r="CQ14" t="inlineStr">
         <is>
-          <t>Moderately connected</t>
+          <t>Not at all connected</t>
         </is>
       </c>
     </row>

</xml_diff>